<commit_message>
Build tag filters from unique sheet tags; comma-separated tags
The Featured filter dropdown was built from a hardcoded TOPICS array, so
any tag not in that list (e.g. Sports) never appeared no matter how many
posts used it. Now both Featured and Projects derive the dropdown from the
unique Tags actually present in the sheet.

- featured.js / projects.js: parse tags on commas only, so multi-word tags
  like 'Clean Energy' stay intact instead of splitting into 'Clean'+'Energy'
- featured.js: dropdown built from unique sheet tags (was TOPICS.filter)
- fetch.xlsx: featured 'Winners' row tag 'Aerospace Entrepreneurship' ->
  'Aerospace, Entrepreneurship' (edited in-place at the cell level so all
  formula cached values elsewhere in the workbook are preserved)
</commit_message>
<xml_diff>
--- a/fetch.xlsx
+++ b/fetch.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ghz\Documents\Claude\Projects\0) VC.Perera - Online Porfoilio\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ghz\Documents\Claude\Projects\000 Online Portfolio - vcperera\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60E439E5-BAD7-42AF-A47F-2854F90BDD6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1568225-6772-4A19-8F6A-B60F65DB8F3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="personas" sheetId="1" r:id="rId1"/>
@@ -3199,7 +3199,7 @@
         <v>231</v>
       </c>
       <c r="E3" t="s">
-        <v>232</v>
+        <v>216</v>
       </c>
       <c r="F3" t="s">
         <v>223</v>
@@ -3323,7 +3323,7 @@
         <v>240</v>
       </c>
       <c r="E8" t="s">
-        <v>232</v>
+        <v>383</v>
       </c>
       <c r="F8" t="s">
         <v>410</v>
@@ -4882,8 +4882,10 @@
       <c r="E2" t="s">
         <v>358</v>
       </c>
-      <c r="F2" t="s">
-        <v>232</v>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Aerospace, Entrepreneurship</t>
+        </is>
       </c>
       <c r="G2" t="s">
         <v>219</v>

</xml_diff>

<commit_message>
Featured update; mobile accolades hi-res viewer + renders; project modal fit
</commit_message>
<xml_diff>
--- a/fetch.xlsx
+++ b/fetch.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ghz\Documents\Claude\Projects\000 Online Portfolio - vcperera\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1568225-6772-4A19-8F6A-B60F65DB8F3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2C4F7C6-A520-4B75-8B72-F844651C5924}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="personas" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="744" uniqueCount="420">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="751" uniqueCount="425">
   <si>
     <t>ID</t>
   </si>
@@ -452,6 +452,9 @@
     <t>Remote</t>
   </si>
   <si>
+    <t>An international content agency serving clients across multiple industries such as Tourism, Tech, and Entertainment. Researched and delivered over 100+ SEO articles, blogs, and marketing copies to drive engagement.</t>
+  </si>
+  <si>
     <t>Axle Global</t>
   </si>
   <si>
@@ -470,6 +473,9 @@
     <t>Hybrid</t>
   </si>
   <si>
+    <t>A startup specialized in digital transformation. Close partners with the Founder, helping revitalize the digital landscapes of our clientele through engaging Web and SEO content that improves conversion rates.</t>
+  </si>
+  <si>
     <t>Third Space Global</t>
   </si>
   <si>
@@ -494,6 +500,9 @@
     <t>Online</t>
   </si>
   <si>
+    <t>An Ed-Tech platform delivering student-centric, 1-to-1 online tutoring for primary and pre-schoolers in the UK. Excelled in balancing young learners' emotional wellbeing, theroetical understanding and timely syllabus execution.</t>
+  </si>
+  <si>
     <t>SEDS KDU</t>
   </si>
   <si>
@@ -515,6 +524,9 @@
     <t>On-site</t>
   </si>
   <si>
+    <t>A dedicated local chapter of a global student-based space organization, designed to foster future aerospace talent and space exploration enthusiasts. Established #TheSpaceForce out of a profound passion for all things Space.</t>
+  </si>
+  <si>
     <t>SEDS Sri Lanka</t>
   </si>
   <si>
@@ -527,6 +539,9 @@
     <t>Mar 2024</t>
   </si>
   <si>
+    <t>Sri Lanka's largest student-based space organization, with a network of local chapters across universities and schools. The Board of Directors &amp; Staff coordinated and drove key national and international outreach initiatives.</t>
+  </si>
+  <si>
     <t>SriLankan Airlines</t>
   </si>
   <si>
@@ -561,6 +576,9 @@
   </si>
   <si>
     <t>Present</t>
+  </si>
+  <si>
+    <t>A French multinational aviation corporation based in Dubai, operating under EASA Part 21J (DOA), 21G (POA), and Part 145 (AMO) approvals. Joined full-time six months prior to graduation, serving as a Design Industrialization Engineer.</t>
   </si>
   <si>
     <t>Satocci</t>
@@ -698,47 +716,13 @@
     <t>Aerospace</t>
   </si>
   <si>
-    <t>Project 1/1-1.webp</t>
-  </si>
-  <si>
-    <t>Project 1/1-1.webp|Project 1/1-2.webp|Project 1/1-3.webp|Project 1/1-4.webp</t>
+    <t>Project 7/7-1.webp</t>
+  </si>
+  <si>
+    <t>Project 7/7-1.webp|Project 7/7-2.webp|Project 7/7-3.webp|Project 7/7-4.webp</t>
   </si>
   <si>
     <t>NO</t>
-  </si>
-  <si>
-    <t>Aerodynamics of a Nano-Coated Airfoil 1/2</t>
-  </si>
-  <si>
-    <t>Numeric Approach (CFD) | Winner: Best Research Project (2024), Department of Aeronautical Engineering</t>
-  </si>
-  <si>
-    <t>Superhydrophobic Surfaces are still cool. In Project 1, the novel study discovered that the superhydrophobic surface properties had
-a positive impact on the overall aerodynamics of the flat plate and the relationship of aerodynamics with the coated area was non-linear. How would it fair with the aerodynamic body being an Airfoil? Would it have more exaggerated effects?
-In this secondary study I used OpenFOAM and SolidWorks to assess the aerodynamics of a NACA 4412 Airfoil, bearing the same principle
-mode of analysis as in Project #1, but for multiple Angles of Attack. Once again, superhydrophobic airfoils, especially those that are partially superhydrophobic, outperformed conventional uncoated airfoils and fully superhydrophobic airfoils.</t>
-  </si>
-  <si>
-    <t>Project 2/2-1.webp</t>
-  </si>
-  <si>
-    <t>YES</t>
-  </si>
-  <si>
-    <t>Aerodynamics of a Nano-Coated Airfoil 2/2</t>
-  </si>
-  <si>
-    <t>Experimental Approach (Lab) | Grant of LKR 1Mn Approved by Combinatorial Advanced Research &amp; Education (KDU-CARE)</t>
-  </si>
-  <si>
-    <t>Yes. Superhydrophobic surfaces are still cool as they were. Projects 1 and 2 had proved that there are positive benefits of
-changing the surface properties of aerodynamic bodies at the nanoscale, but these were virtual simulations. The next step was to
-perform Project 2 under lab conditions to observe how superhydrophobic surfaces perform aerodynamically in a real-world scenario.
-The experimental design, value proposition, budgetary requirements and timeline was pitched to the heads of faculties and
-representatives of KDU-CARE. It was decided that a research grant of 1 Million LKR would be awarded, however, due to administrative delays, the project did not kickoff and was paused indefinitely.</t>
-  </si>
-  <si>
-    <t>Project 3/3-1.webp</t>
   </si>
   <si>
     <t>Aerodynamics of a Nano-Coated Flat Plate</t>
@@ -755,7 +739,44 @@
 helped analyze what the most optimal degree of coating would be to achieve the best aerodynamics possible.</t>
   </si>
   <si>
-    <t>Aerospace Entrepreneurship</t>
+    <t>Project 6/6-1.webp</t>
+  </si>
+  <si>
+    <t>Project 6/6-1.webp|Project 6/6-2.webp|Project 6/6-3.webp|Project 6/6-4.webp|Project 6/6-5.webp|Project 6/6-6.webp|Project 6/6-7.webp|Project 6/6-8.webp</t>
+  </si>
+  <si>
+    <t>YES</t>
+  </si>
+  <si>
+    <t>Aerodynamics of a Nano-Coated Airfoil 1/2</t>
+  </si>
+  <si>
+    <t>Numeric Approach (CFD) | Winner: Best Research Project (2024), Department of Aeronautical Engineering</t>
+  </si>
+  <si>
+    <t>Superhydrophobic Surfaces are still cool. In Project 1, the novel study discovered that the superhydrophobic surface properties had
+a positive impact on the overall aerodynamics of the flat plate and the relationship of aerodynamics with the coated area was non-linear. How would it fair with the aerodynamic body being an Airfoil? Would it have more exaggerated effects?
+In this secondary study I used OpenFOAM and SolidWorks to assess the aerodynamics of a NACA 4412 Airfoil, bearing the same principle
+mode of analysis as in Project #1, but for multiple Angles of Attack. Once again, superhydrophobic airfoils, especially those that are partially superhydrophobic, outperformed conventional uncoated airfoils and fully superhydrophobic airfoils.</t>
+  </si>
+  <si>
+    <t>Project 5/5-1.webp</t>
+  </si>
+  <si>
+    <t>Project 5/5-1.webp|Project 5/5-2.webp|Project 5/5-3.webp|Project 5/5-4.webp|Project 5/5-5.webp</t>
+  </si>
+  <si>
+    <t>Aerodynamics of a Nano-Coated Airfoil 2/2</t>
+  </si>
+  <si>
+    <t>Experimental Approach (Lab) | Grant of LKR 1Mn Approved by Combinatorial Advanced Research &amp; Education (KDU-CARE)</t>
+  </si>
+  <si>
+    <t>Yes. Superhydrophobic surfaces are still cool as they were. Projects 1 and 2 had proved that there are positive benefits of
+changing the surface properties of aerodynamic bodies at the nanoscale, but these were virtual simulations. The next step was to
+perform Project 2 under lab conditions to observe how superhydrophobic surfaces perform aerodynamically in a real-world scenario.
+The experimental design, value proposition, budgetary requirements and timeline was pitched to the heads of faculties and
+representatives of KDU-CARE. It was decided that a research grant of 1 Million LKR would be awarded, however, due to administrative delays, the project did not kickoff and was paused indefinitely.</t>
   </si>
   <si>
     <t>Project 4/4-1.webp</t>
@@ -767,10 +788,19 @@
     <t>Designing a Jet Engine from scratch using a 2D Draft as a Sketch Picture</t>
   </si>
   <si>
-    <t>Project 5/5-1.webp</t>
-  </si>
-  <si>
-    <t>Project 5/5-1.webp|Project 5/5-2.webp</t>
+    <t>Project 3/3-1.webp</t>
+  </si>
+  <si>
+    <t>Project 3/3-1.webp|Project 3/3-2.webp</t>
+  </si>
+  <si>
+    <t>Developing a 3D Model of an A380</t>
+  </si>
+  <si>
+    <t>Designing an A380 exterior from scratch using a 2D Draft as a Sketch Picture</t>
+  </si>
+  <si>
+    <t>Project 2/2-1.webp</t>
   </si>
   <si>
     <t>HYDRATech: Local Nanocoating Production</t>
@@ -785,7 +815,13 @@
 to make it through to the final stage due to the Capital Intensive nature of the project.</t>
   </si>
   <si>
-    <t>Project 6/6-1.webp</t>
+    <t>Entrepreneurship</t>
+  </si>
+  <si>
+    <t>Project 1/1-1.webp</t>
+  </si>
+  <si>
+    <t>Project 1/1-1.webp|Project 1/1-2.webp|Project 1/1-3.webp</t>
   </si>
   <si>
     <t>Issuer</t>
@@ -860,6 +896,9 @@
     <t>https://www.coursera.org/account/accomplishments/verify/2NZXDQTQWSA7</t>
   </si>
   <si>
+    <t>Best Research Project</t>
+  </si>
+  <si>
     <t>Kotelawala Defense University</t>
   </si>
   <si>
@@ -1127,199 +1166,175 @@
     <t>Post_Link</t>
   </si>
   <si>
+    <t>thumbs/14.webp</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/posts/the-futures-forum_spaceungana2026-spacefuturesforum-nextgenleaders-activity-7484926325519134720-dpOL?utm_source=share&amp;utm_medium=member_desktop&amp;rcm=ACoAADSwLqIBLzQLDm-Klx9wMM6NKZChtEvLQUo</t>
+  </si>
+  <si>
     <t>Winners: Space Entrepreneurship Challenge</t>
   </si>
   <si>
     <t>5th Edition organized by EIIS with Airbus D&amp;S, tied to the Master of Arts in Space Entrepreneurship.</t>
   </si>
   <si>
+    <t>thumbs/13.webp</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/posts/melodi-askelof_innovation-resilience-execution-activity-7460594246371434496-iSyu?utm_source=share&amp;utm_medium=member_desktop&amp;rcm=ACoAADSwLqIBLzQLDm-Klx9wMM6NKZChtEvLQUo</t>
+  </si>
+  <si>
+    <t>Aerospace, Entrepreneurship</t>
+  </si>
+  <si>
+    <t>Recognised as the Best Overall Local Chapter by SEDS Sri Lanka, within two years of its inception.</t>
+  </si>
+  <si>
+    <t>thumbs/12.webp</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/posts/seds-kdu_sedskdu-bestoverallchapter-teamwork-activity-7315058728968286208-UoCm?utm_source=social_share_send&amp;utm_medium=android_app&amp;rcm=ACoAADSwLqIBLzQLDm-Klx9wMM6NKZChtEvLQUo&amp;utm_campaign=copy_link</t>
+  </si>
+  <si>
+    <t>Vishal Appointed as Chairperson of SEDS SL</t>
+  </si>
+  <si>
+    <t>Leading the 7th Board of Directors and Board of Staff of SEDS Sri Lanka (2024/25).</t>
+  </si>
+  <si>
+    <t>thumbs/11.webp</t>
+  </si>
+  <si>
+    <t>https://foe.kdu.ac.lk/aero/2024/04/18/vishal-perera-appointed-as-chairperson-seds-sri-lanka-39</t>
+  </si>
+  <si>
+    <t>Awarded by the Department of Aeronautical Engineering at the Final Year Exhibition, KDU.</t>
+  </si>
+  <si>
+    <t>thumbs/10.webp</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/p/C4Vd0d1REmQ/?igsh=MWw1YTY1emcxcDM5Yg==</t>
+  </si>
+  <si>
+    <t>Congratulations: Vishal Perera of SEDS KDU!</t>
+  </si>
+  <si>
+    <t>Congratulatory post by SEDS KDU for the role ahead as National Chairperson.</t>
+  </si>
+  <si>
+    <t>thumbs/9.webp</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/p/C4Sr1ssxqcH/?igsh=MXVidWI1OTRlZG9pcQ==</t>
+  </si>
+  <si>
+    <t>Introducing the Chairperson of SEDS SL</t>
+  </si>
+  <si>
+    <t>Introductory Feature on the newly appointed Board of Directors of SEDS Sri Lanka, 2024-25.</t>
+  </si>
+  <si>
+    <t>thumbs/8.webp</t>
+  </si>
+  <si>
+    <t>https://foe.kdu.ac.lk/aero/2022/08/13/formation-of-the-space-force-27</t>
+  </si>
+  <si>
+    <t>Formation of the “Space Force”</t>
+  </si>
+  <si>
+    <t>Article on the formation of the SEDS KDU Local Chapter as the Founding Board.</t>
+  </si>
+  <si>
+    <t>thumbs/7.webp</t>
+  </si>
+  <si>
+    <t>https://foe.kdu.ac.lk/aero/2024/01/24/final-year-project-exhibition-2024-35</t>
+  </si>
+  <si>
+    <t>Semi Finalists: IEEE Innovation Nation SL</t>
+  </si>
+  <si>
+    <t>Conceptualizing a startup aiming to produce nanotech based coatings, locally.</t>
+  </si>
+  <si>
+    <t>thumbs/6.webp</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/IEEEINSL/posts/here-we-present-to-you-the-most-talented-semi-finalists-whose-hard-work-dedicati/3027737500833258/</t>
+  </si>
+  <si>
+    <t>Winners: Pentathlon 2022</t>
+  </si>
+  <si>
+    <t>An inter-university article-writing competition hosted by MoraSpirit, a premier sports network.</t>
+  </si>
+  <si>
+    <t>thumbs/5.webp</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/MoraSpirit/posts/after-a-close-competition-between-all-the-participants-we-are-pleased-to-inform-/424187246412243/</t>
+  </si>
+  <si>
+    <t>Climate Crisis and Clean Energy</t>
+  </si>
+  <si>
+    <t>Article on the Severity of the Climate Crisis. Competition organized by the IEEE SLTC.</t>
+  </si>
+  <si>
+    <t>thumbs/4.webp</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/photo?fbid=1106724503145581&amp;set=a.1106720086479356</t>
+  </si>
+  <si>
+    <t>Clean Energy</t>
+  </si>
+  <si>
+    <t>Top 8: Most Popular Schoolboy Cricketers</t>
+  </si>
+  <si>
+    <t>batsman.lk nominee based on performers at the All-Island School's Cricket Tournament (D2) 2019</t>
+  </si>
+  <si>
+    <t>thumbs/3.webp</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/reel/2660611044253733</t>
+  </si>
+  <si>
+    <t>Stats Alert: 176 Runs vs Royal Panadura</t>
+  </si>
+  <si>
+    <t>"Vishal Perera's 176 was the highlight for the Wattala boys in that game."</t>
+  </si>
+  <si>
+    <t>thumbs/2.webp</t>
+  </si>
+  <si>
+    <t>https://www.thepapare.com/u19-schools-cricket-division-2-1st-week-of-january-2020-roundup/</t>
+  </si>
+  <si>
+    <t>Daily News: 176 Runs vs Royal Panadura</t>
+  </si>
+  <si>
+    <t>"Vishal Perera skipper and right hand opener of LISW scored 176 runs in 202 balls…"</t>
+  </si>
+  <si>
     <t>thumbs/1.webp</t>
   </si>
   <si>
-    <t>https://www.linkedin.com/posts/melodi-askelof_innovation-resilience-execution-activity-7460594246371434496-iSyu?utm_source=share&amp;utm_medium=member_desktop&amp;rcm=ACoAADSwLqIBLzQLDm-Klx9wMM6NKZChtEvLQUo</t>
-  </si>
-  <si>
-    <t>SEDS SL's Best Local Chapter</t>
-  </si>
-  <si>
-    <t>thumbs/2.webp</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/posts/seds-kdu_sedskdu-bestoverallchapter-teamwork-activity-7315058728968286208-UoCm?utm_source=social_share_send&amp;utm_medium=android_app&amp;rcm=ACoAADSwLqIBLzQLDm-Klx9wMM6NKZChtEvLQUo&amp;utm_campaign=copy_link</t>
-  </si>
-  <si>
-    <t>Vishal Appointed as Chairperson of SEDS SL</t>
-  </si>
-  <si>
-    <t>thumbs/3.webp</t>
-  </si>
-  <si>
-    <t>https://foe.kdu.ac.lk/aero/2024/04/18/vishal-perera-appointed-as-chairperson-seds-sri-lanka-39</t>
-  </si>
-  <si>
-    <t>Best Research Project</t>
-  </si>
-  <si>
-    <t>Awarded by the Department of Aeronautical Engineering at the Final Year Exhibition, KDU.</t>
-  </si>
-  <si>
-    <t>thumbs/4.webp</t>
-  </si>
-  <si>
-    <t>https://www.instagram.com/p/C4Vd0d1REmQ/?igsh=MWw1YTY1emcxcDM5Yg==</t>
-  </si>
-  <si>
-    <t>Congratulations: Vishal Perera of SEDS KDU!</t>
-  </si>
-  <si>
-    <t>Congratulatory post by SEDS KDU for the role ahead as National Chairperson.</t>
-  </si>
-  <si>
-    <t>thumbs/5.webp</t>
-  </si>
-  <si>
-    <t>https://www.instagram.com/p/C4Sr1ssxqcH/?igsh=MXVidWI1OTRlZG9pcQ==</t>
-  </si>
-  <si>
-    <t>Introducing the Chairperson of SEDS SL</t>
-  </si>
-  <si>
-    <t>Introductory Feature on the newly appointed Board of Directors of SEDS Sri Lanka, 2024-25.</t>
-  </si>
-  <si>
-    <t>thumbs/6.webp</t>
-  </si>
-  <si>
-    <t>https://foe.kdu.ac.lk/aero/2022/08/13/formation-of-the-space-force-27</t>
-  </si>
-  <si>
-    <t>Article on the formation of the SEDS KDU Local Chapter as the Founding Board.</t>
-  </si>
-  <si>
-    <t>thumbs/7.webp</t>
-  </si>
-  <si>
-    <t>https://foe.kdu.ac.lk/aero/2024/01/24/final-year-project-exhibition-2024-35</t>
-  </si>
-  <si>
-    <t>Conceptualizing a startup aiming to produce nanotech based coatings, locally.</t>
-  </si>
-  <si>
-    <t>thumbs/8.webp</t>
-  </si>
-  <si>
-    <t>https://www.facebook.com/IEEEINSL/posts/here-we-present-to-you-the-most-talented-semi-finalists-whose-hard-work-dedicati/3027737500833258/</t>
-  </si>
-  <si>
-    <t>Entrepreneurship</t>
-  </si>
-  <si>
-    <t>Winners: Pentathlon 2022</t>
-  </si>
-  <si>
-    <t>An inter-university article-writing competition hosted by MoraSpirit, a premier sports network.</t>
-  </si>
-  <si>
-    <t>thumbs/9.webp</t>
-  </si>
-  <si>
-    <t>https://www.facebook.com/MoraSpirit/posts/after-a-close-competition-between-all-the-participants-we-are-pleased-to-inform-/424187246412243/</t>
-  </si>
-  <si>
-    <t>Climate Crisis and Clean Energy</t>
-  </si>
-  <si>
-    <t>Article on the Severity of the Climate Crisis. Competition organized by the IEEE SLTC.</t>
-  </si>
-  <si>
-    <t>thumbs/10.webp</t>
-  </si>
-  <si>
-    <t>https://www.facebook.com/photo?fbid=1106724503145581&amp;set=a.1106720086479356</t>
-  </si>
-  <si>
-    <t>Clean Energy</t>
-  </si>
-  <si>
-    <t>batsman.lk nominee based on performers at the All-Island School's Cricket Tournament (D2) 2019</t>
-  </si>
-  <si>
-    <t>thumbs/11.webp</t>
-  </si>
-  <si>
-    <t>https://www.facebook.com/reel/2660611044253733</t>
-  </si>
-  <si>
-    <t>thumbs/12.webp</t>
-  </si>
-  <si>
-    <t>https://www.thepapare.com/u19-schools-cricket-division-2-1st-week-of-january-2020-roundup/</t>
-  </si>
-  <si>
-    <t>Daily News: 176 Runs vs Royal Panadura</t>
-  </si>
-  <si>
-    <t>thumbs/13.webp</t>
-  </si>
-  <si>
-    <t>Formation of the “Space Force”</t>
-  </si>
-  <si>
-    <t>Semi Finalists: IEEE Innovation Nation SL</t>
-  </si>
-  <si>
-    <t>Top 8: Most Popular Schoolboy Cricketers</t>
-  </si>
-  <si>
-    <t>Stats Alert: 176 Runs vs Royal Panadura</t>
-  </si>
-  <si>
-    <t>"Vishal Perera skipper and right hand opener of LISW scored 176 runs in 202 balls…"</t>
-  </si>
-  <si>
-    <t>"Vishal Perera's 176 was the highlight for the Wattala boys in that game."</t>
-  </si>
-  <si>
-    <t>Leading the 7th Board of Directors and Board of Staff of SEDS Sri Lanka (2024/25).</t>
-  </si>
-  <si>
-    <t>Recognised as the Best Overall Local Chapter by SEDS Sri Lanka, within two years of its inception.</t>
-  </si>
-  <si>
-    <t>Developing a 3D Model of an A380</t>
-  </si>
-  <si>
-    <t>Designing an A380 exterior from scratch using a 2D Draft as a Sketch Picture</t>
-  </si>
-  <si>
-    <t>Project 7/7-1.webp</t>
-  </si>
-  <si>
-    <t>Project 2/2-1.webp|Project 2/2-2.webp|Project 2/2-3.webp|Project 2/2-4.webp|Project 2/2-5.webp|Project 2/2-6.webp|Project 2/2-7.webp|Project 2/2-8.webp</t>
-  </si>
-  <si>
-    <t>Project 3/3-1.webp|Project 3/3-2.webp|Project 3/3-3.webp|Project 3/3-4.webp|Project 3/3-5.webp</t>
-  </si>
-  <si>
-    <t>Project 7/7-1.webp|Project 7/7-2.webp|Project 7/7-3.webp</t>
-  </si>
-  <si>
-    <t>An international content agency serving clients across multiple industries such as Tourism, Tech, and Entertainment. Researched and delivered over 100+ SEO articles, blogs, and marketing copies to drive engagement.</t>
-  </si>
-  <si>
-    <t>A startup specialized in digital transformation. Close partners with the Founder, helping revitalize the digital landscapes of our clientele through engaging Web and SEO content that improves conversion rates.</t>
-  </si>
-  <si>
-    <t>An Ed-Tech platform delivering student-centric, 1-to-1 online tutoring for primary and pre-schoolers in the UK. Excelled in balancing young learners' emotional wellbeing, theroetical understanding and timely syllabus execution.</t>
-  </si>
-  <si>
-    <t>A dedicated local chapter of a global student-based space organization, designed to foster future aerospace talent and space exploration enthusiasts. Established #TheSpaceForce out of a profound passion for all things Space.</t>
-  </si>
-  <si>
-    <t>Sri Lanka's largest student-based space organization, with a network of local chapters across universities and schools. The Board of Directors &amp; Staff coordinated and drove key national and international outreach initiatives.</t>
-  </si>
-  <si>
-    <t>A French multinational aviation corporation based in Dubai, operating under EASA Part 21J (DOA), 21G (POA), and Part 145 (AMO) approvals. Joined full-time six months prior to graduation, serving as a Design Industrialization Engineer.</t>
+    <t>Africa's premier virtual forum on space futures, innovation and collaboration.</t>
+  </si>
+  <si>
+    <t>Distinguished Panelist: SPACE UNGANA '26</t>
+  </si>
+  <si>
+    <t>SEDS KDU: SEDS SL's Best Local Chapter</t>
+  </si>
+  <si>
+    <t>Best Research Project: Aero Engineering</t>
   </si>
 </sst>
 </file>
@@ -2711,7 +2726,7 @@
         <v>135</v>
       </c>
       <c r="J2" t="s">
-        <v>414</v>
+        <v>136</v>
       </c>
       <c r="K2">
         <v>2.468</v>
@@ -2722,13 +2737,13 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C3" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D3" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E3" t="s">
         <v>131</v>
@@ -2737,16 +2752,16 @@
         <v>132</v>
       </c>
       <c r="G3" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="H3" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="I3" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="J3" t="s">
-        <v>415</v>
+        <v>143</v>
       </c>
       <c r="K3">
         <v>2.5</v>
@@ -2757,31 +2772,31 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C4" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="D4" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="E4" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="F4" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="G4" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="H4" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="I4" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="J4" t="s">
-        <v>416</v>
+        <v>152</v>
       </c>
       <c r="K4">
         <v>2.75</v>
@@ -2792,31 +2807,31 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="C5" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="D5" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="E5" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="F5" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="G5" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="H5" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="I5" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="J5" t="s">
-        <v>417</v>
+        <v>160</v>
       </c>
       <c r="K5">
         <v>2.3050000000000002</v>
@@ -2827,31 +2842,31 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="C6" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="D6" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="E6" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="F6" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="G6" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="H6" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="I6" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="J6" t="s">
-        <v>418</v>
+        <v>165</v>
       </c>
       <c r="K6">
         <v>2.7629999999999999</v>
@@ -2862,31 +2877,31 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="C7" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="D7" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="E7" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="F7" t="s">
+        <v>169</v>
+      </c>
+      <c r="G7" t="s">
+        <v>170</v>
+      </c>
+      <c r="H7" t="s">
         <v>164</v>
       </c>
-      <c r="G7" t="s">
-        <v>165</v>
-      </c>
-      <c r="H7" t="s">
-        <v>160</v>
-      </c>
       <c r="I7" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="J7" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="K7">
         <v>3.5</v>
@@ -2897,31 +2912,31 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="C8" t="s">
+        <v>173</v>
+      </c>
+      <c r="D8" t="s">
+        <v>174</v>
+      </c>
+      <c r="E8" t="s">
         <v>168</v>
       </c>
-      <c r="D8" t="s">
-        <v>169</v>
-      </c>
-      <c r="E8" t="s">
-        <v>163</v>
-      </c>
       <c r="F8" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="G8" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="H8" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="I8" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="J8" t="s">
-        <v>419</v>
+        <v>178</v>
       </c>
       <c r="K8">
         <v>0.75</v>
@@ -2932,31 +2947,31 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="C9" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="D9" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="E9" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="F9" t="s">
-        <v>177</v>
+        <v>183</v>
       </c>
       <c r="G9" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
       <c r="H9" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="I9" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="J9" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="K9">
         <v>2.75</v>
@@ -2967,31 +2982,31 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
       <c r="C10" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="D10" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="E10" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="F10" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="G10" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="H10" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="I10" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="J10" t="s">
-        <v>186</v>
+        <v>192</v>
       </c>
       <c r="K10">
         <v>3.7469999999999999</v>
@@ -3022,16 +3037,16 @@
         <v>1</v>
       </c>
       <c r="D1" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
       <c r="E1" t="s">
         <v>126</v>
       </c>
       <c r="F1" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="G1" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="H1" t="s">
         <v>22</v>
@@ -3042,22 +3057,22 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="C2" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="D2" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="E2" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="F2" t="s">
-        <v>194</v>
+        <v>200</v>
       </c>
       <c r="G2" t="s">
-        <v>195</v>
+        <v>201</v>
       </c>
       <c r="H2">
         <v>2.5</v>
@@ -3068,22 +3083,22 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>196</v>
+        <v>202</v>
       </c>
       <c r="C3" t="s">
-        <v>197</v>
+        <v>203</v>
       </c>
       <c r="D3" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
       <c r="E3" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="F3" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="G3" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
       <c r="H3">
         <v>3</v>
@@ -3094,22 +3109,22 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>202</v>
+        <v>208</v>
       </c>
       <c r="C4" t="s">
-        <v>203</v>
+        <v>209</v>
       </c>
       <c r="D4" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
       <c r="E4" t="s">
-        <v>205</v>
+        <v>211</v>
       </c>
       <c r="F4" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="G4" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
       <c r="H4">
         <v>3</v>
@@ -3138,22 +3153,22 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="C1" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="D1" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="E1" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
       <c r="F1" t="s">
-        <v>211</v>
+        <v>217</v>
       </c>
       <c r="G1" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="H1" t="s">
         <v>22</v>
@@ -3161,80 +3176,80 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="B2" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="C2" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="D2" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="E2" t="s">
-        <v>216</v>
+        <v>222</v>
       </c>
       <c r="F2" t="s">
-        <v>217</v>
+        <v>223</v>
       </c>
       <c r="G2" t="s">
-        <v>218</v>
+        <v>224</v>
       </c>
       <c r="H2" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="B3" t="s">
+        <v>226</v>
+      </c>
+      <c r="C3" t="s">
+        <v>227</v>
+      </c>
+      <c r="D3" t="s">
+        <v>228</v>
+      </c>
+      <c r="E3" t="s">
+        <v>222</v>
+      </c>
+      <c r="F3" t="s">
         <v>229</v>
       </c>
-      <c r="C3" t="s">
+      <c r="G3" t="s">
         <v>230</v>
       </c>
-      <c r="D3" t="s">
+      <c r="H3" t="s">
         <v>231</v>
-      </c>
-      <c r="E3" t="s">
-        <v>216</v>
-      </c>
-      <c r="F3" t="s">
-        <v>223</v>
-      </c>
-      <c r="G3" t="s">
-        <v>411</v>
-      </c>
-      <c r="H3" t="s">
-        <v>224</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>220</v>
+        <v>232</v>
       </c>
       <c r="C4" t="s">
-        <v>221</v>
+        <v>233</v>
       </c>
       <c r="D4" t="s">
+        <v>234</v>
+      </c>
+      <c r="E4" t="s">
         <v>222</v>
       </c>
-      <c r="E4" t="s">
-        <v>216</v>
-      </c>
       <c r="F4" t="s">
-        <v>228</v>
+        <v>235</v>
       </c>
       <c r="G4" t="s">
-        <v>412</v>
+        <v>236</v>
       </c>
       <c r="H4" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.35">
@@ -3242,97 +3257,97 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>225</v>
+        <v>237</v>
       </c>
       <c r="C5" t="s">
-        <v>226</v>
+        <v>238</v>
       </c>
       <c r="D5" t="s">
-        <v>227</v>
+        <v>239</v>
       </c>
       <c r="E5" t="s">
-        <v>216</v>
+        <v>222</v>
       </c>
       <c r="F5" t="s">
-        <v>233</v>
+        <v>240</v>
       </c>
       <c r="G5" t="s">
-        <v>228</v>
+        <v>235</v>
       </c>
       <c r="H5" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B6" t="s">
-        <v>234</v>
+        <v>241</v>
       </c>
       <c r="C6" t="s">
-        <v>235</v>
+        <v>242</v>
       </c>
       <c r="E6" t="s">
-        <v>216</v>
+        <v>222</v>
       </c>
       <c r="F6" t="s">
-        <v>236</v>
+        <v>243</v>
       </c>
       <c r="G6" t="s">
-        <v>237</v>
+        <v>244</v>
       </c>
       <c r="H6" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="B7" t="s">
-        <v>408</v>
+        <v>245</v>
       </c>
       <c r="C7" t="s">
-        <v>409</v>
+        <v>246</v>
       </c>
       <c r="E7" t="s">
-        <v>216</v>
+        <v>222</v>
       </c>
       <c r="F7" t="s">
-        <v>241</v>
+        <v>247</v>
       </c>
       <c r="G7" t="s">
-        <v>241</v>
+        <v>247</v>
       </c>
       <c r="H7" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="B8" t="s">
-        <v>238</v>
+        <v>248</v>
       </c>
       <c r="C8" t="s">
-        <v>239</v>
+        <v>249</v>
       </c>
       <c r="D8" t="s">
-        <v>240</v>
+        <v>250</v>
       </c>
       <c r="E8" t="s">
-        <v>383</v>
+        <v>251</v>
       </c>
       <c r="F8" t="s">
-        <v>410</v>
+        <v>252</v>
       </c>
       <c r="G8" t="s">
-        <v>413</v>
+        <v>253</v>
       </c>
       <c r="H8" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
     </row>
   </sheetData>
@@ -3360,25 +3375,25 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="C1" t="s">
-        <v>242</v>
+        <v>254</v>
       </c>
       <c r="D1" t="s">
-        <v>243</v>
+        <v>255</v>
       </c>
       <c r="E1" t="s">
-        <v>211</v>
+        <v>217</v>
       </c>
       <c r="F1" t="s">
-        <v>244</v>
+        <v>256</v>
       </c>
       <c r="G1" t="s">
-        <v>245</v>
+        <v>257</v>
       </c>
       <c r="H1" t="s">
-        <v>246</v>
+        <v>258</v>
       </c>
       <c r="I1" t="s">
         <v>22</v>
@@ -3389,27 +3404,27 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>247</v>
+        <v>259</v>
       </c>
       <c r="C2" t="s">
-        <v>248</v>
+        <v>260</v>
       </c>
       <c r="E2" t="str">
-        <f t="shared" ref="E2" si="0">"thumbs/" &amp; B2 &amp; ".webp"</f>
+        <f t="shared" ref="E2:E33" si="0">"thumbs/" &amp; B2 &amp; ".webp"</f>
         <v>thumbs/Master of Arts - Space Entrepreneurship.webp</v>
       </c>
       <c r="F2" t="str">
-        <f t="shared" ref="F2" si="1">"pdfs/" &amp; B2 &amp; ".pdf"</f>
+        <f t="shared" ref="F2:F33" si="1">"pdfs/" &amp; B2 &amp; ".pdf"</f>
         <v>pdfs/Master of Arts - Space Entrepreneurship.pdf</v>
       </c>
       <c r="G2" t="s">
-        <v>249</v>
+        <v>261</v>
       </c>
       <c r="H2" t="s">
-        <v>248</v>
+        <v>260</v>
       </c>
       <c r="I2" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.35">
@@ -3417,24 +3432,24 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>250</v>
+        <v>262</v>
       </c>
       <c r="C3" t="s">
-        <v>248</v>
+        <v>260</v>
       </c>
       <c r="E3" t="str">
-        <f t="shared" ref="E3:E52" si="2">"thumbs/" &amp; B3 &amp; ".webp"</f>
+        <f t="shared" si="0"/>
         <v>thumbs/Acceptance Letter - EIIS.webp</v>
       </c>
       <c r="F3" t="str">
-        <f t="shared" ref="F3:F52" si="3">"pdfs/" &amp; B3 &amp; ".pdf"</f>
+        <f t="shared" si="1"/>
         <v>pdfs/Acceptance Letter - EIIS.pdf</v>
       </c>
       <c r="G3" t="s">
-        <v>249</v>
+        <v>261</v>
       </c>
       <c r="H3" t="s">
-        <v>248</v>
+        <v>260</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.35">
@@ -3442,30 +3457,30 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>251</v>
+        <v>263</v>
       </c>
       <c r="C4" t="s">
-        <v>252</v>
+        <v>264</v>
       </c>
       <c r="D4" t="s">
-        <v>253</v>
+        <v>265</v>
       </c>
       <c r="E4" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>thumbs/Digitalisation in Aeronautics.webp</v>
       </c>
       <c r="F4" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>pdfs/Digitalisation in Aeronautics.pdf</v>
       </c>
       <c r="G4" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="H4" t="s">
-        <v>255</v>
+        <v>267</v>
       </c>
       <c r="I4" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.35">
@@ -3473,30 +3488,30 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>256</v>
+        <v>268</v>
       </c>
       <c r="C5" t="s">
-        <v>252</v>
+        <v>264</v>
       </c>
       <c r="D5" t="s">
-        <v>257</v>
+        <v>269</v>
       </c>
       <c r="E5" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>thumbs/Digitalisation in Space Research.webp</v>
       </c>
       <c r="F5" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>pdfs/Digitalisation in Space Research.pdf</v>
       </c>
       <c r="G5" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="H5" t="s">
-        <v>255</v>
+        <v>267</v>
       </c>
       <c r="I5" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.35">
@@ -3504,30 +3519,30 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>258</v>
+        <v>270</v>
       </c>
       <c r="C6" t="s">
-        <v>252</v>
+        <v>264</v>
       </c>
       <c r="D6" t="s">
-        <v>259</v>
+        <v>271</v>
       </c>
       <c r="E6" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>thumbs/Digitalisation in the Aerospace Industry.webp</v>
       </c>
       <c r="F6" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>pdfs/Digitalisation in the Aerospace Industry.pdf</v>
       </c>
       <c r="G6" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="H6" t="s">
-        <v>255</v>
+        <v>267</v>
       </c>
       <c r="I6" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.35">
@@ -3535,27 +3550,27 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>260</v>
+        <v>272</v>
       </c>
       <c r="C7" t="s">
-        <v>261</v>
+        <v>273</v>
       </c>
       <c r="D7" t="s">
-        <v>262</v>
+        <v>274</v>
       </c>
       <c r="E7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>thumbs/Aerospace Materials.webp</v>
       </c>
       <c r="F7" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>pdfs/Aerospace Materials.pdf</v>
       </c>
       <c r="G7" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="I7" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.35">
@@ -3563,27 +3578,27 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>263</v>
+        <v>275</v>
       </c>
       <c r="C8" t="s">
-        <v>264</v>
+        <v>276</v>
       </c>
       <c r="D8" t="s">
-        <v>265</v>
+        <v>277</v>
       </c>
       <c r="E8" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>thumbs/Robotics - Aerial Robotics.webp</v>
       </c>
       <c r="F8" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>pdfs/Robotics - Aerial Robotics.pdf</v>
       </c>
       <c r="G8" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="I8" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.35">
@@ -3591,21 +3606,21 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>365</v>
+        <v>278</v>
       </c>
       <c r="C9" t="s">
-        <v>266</v>
+        <v>279</v>
       </c>
       <c r="E9" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>thumbs/Best Research Project.webp</v>
       </c>
       <c r="F9" t="str">
-        <f>"pdfs/" &amp; B9 &amp; ".pdf"</f>
+        <f t="shared" si="1"/>
         <v>pdfs/Best Research Project.pdf</v>
       </c>
       <c r="I9" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.35">
@@ -3613,24 +3628,24 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>267</v>
+        <v>280</v>
       </c>
       <c r="C10" t="s">
-        <v>268</v>
+        <v>281</v>
       </c>
       <c r="E10" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>thumbs/Best Poster Presentation.webp</v>
       </c>
       <c r="F10" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>pdfs/Best Poster Presentation.pdf</v>
       </c>
       <c r="G10" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="I10" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.35">
@@ -3638,24 +3653,24 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>269</v>
+        <v>282</v>
       </c>
       <c r="C11" t="s">
-        <v>268</v>
+        <v>281</v>
       </c>
       <c r="E11" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>thumbs/Paper Presentation at IRC.webp</v>
       </c>
       <c r="F11" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>pdfs/Paper Presentation at IRC.pdf</v>
       </c>
       <c r="G11" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="I11" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.35">
@@ -3663,27 +3678,27 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>270</v>
+        <v>283</v>
       </c>
       <c r="C12" t="s">
+        <v>279</v>
+      </c>
+      <c r="E12" t="str">
+        <f t="shared" si="0"/>
+        <v>thumbs/BSc. (Hons) Aeronautical Engineering.webp</v>
+      </c>
+      <c r="F12" t="str">
+        <f t="shared" si="1"/>
+        <v>pdfs/BSc. (Hons) Aeronautical Engineering.pdf</v>
+      </c>
+      <c r="G12" t="s">
         <v>266</v>
       </c>
-      <c r="E12" t="str">
-        <f t="shared" si="2"/>
-        <v>thumbs/BSc. (Hons) Aeronautical Engineering.webp</v>
-      </c>
-      <c r="F12" t="str">
-        <f t="shared" si="3"/>
-        <v>pdfs/BSc. (Hons) Aeronautical Engineering.pdf</v>
-      </c>
-      <c r="G12" t="s">
-        <v>254</v>
-      </c>
       <c r="H12" t="s">
-        <v>271</v>
+        <v>284</v>
       </c>
       <c r="I12" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.35">
@@ -3691,27 +3706,27 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>272</v>
+        <v>285</v>
       </c>
       <c r="C13" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="E13" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>thumbs/Chairperson - SEDS SL.webp</v>
       </c>
       <c r="F13" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>pdfs/Chairperson - SEDS SL.pdf</v>
       </c>
       <c r="G13" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="H13" t="s">
-        <v>271</v>
+        <v>284</v>
       </c>
       <c r="I13" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.35">
@@ -3719,24 +3734,24 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>273</v>
+        <v>286</v>
       </c>
       <c r="C14" t="s">
+        <v>279</v>
+      </c>
+      <c r="E14" t="str">
+        <f t="shared" si="0"/>
+        <v>thumbs/President - SEDS KDU.webp</v>
+      </c>
+      <c r="F14" t="str">
+        <f t="shared" si="1"/>
+        <v>pdfs/President - SEDS KDU.pdf</v>
+      </c>
+      <c r="G14" t="s">
         <v>266</v>
       </c>
-      <c r="E14" t="str">
-        <f t="shared" si="2"/>
-        <v>thumbs/President - SEDS KDU.webp</v>
-      </c>
-      <c r="F14" t="str">
-        <f t="shared" si="3"/>
-        <v>pdfs/President - SEDS KDU.pdf</v>
-      </c>
-      <c r="G14" t="s">
-        <v>254</v>
-      </c>
       <c r="I14" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.35">
@@ -3744,24 +3759,24 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>274</v>
+        <v>287</v>
       </c>
       <c r="C15" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="E15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>thumbs/Service Letter.webp</v>
       </c>
       <c r="F15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>pdfs/Service Letter.pdf</v>
       </c>
       <c r="G15" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="I15" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.35">
@@ -3769,27 +3784,27 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>275</v>
+        <v>288</v>
       </c>
       <c r="C16" t="s">
-        <v>276</v>
+        <v>289</v>
       </c>
       <c r="D16" t="s">
-        <v>277</v>
+        <v>290</v>
       </c>
       <c r="E16" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>thumbs/Semi-Finalists - IEEE INSL 2021.webp</v>
       </c>
       <c r="F16" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>pdfs/Semi-Finalists - IEEE INSL 2021.pdf</v>
       </c>
       <c r="G16" t="s">
-        <v>278</v>
+        <v>291</v>
       </c>
       <c r="I16" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.35">
@@ -3797,24 +3812,24 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
+        <v>292</v>
+      </c>
+      <c r="C17" t="s">
         <v>279</v>
       </c>
-      <c r="C17" t="s">
-        <v>266</v>
-      </c>
       <c r="E17" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>thumbs/Inter-Faculty Cricket (2022).webp</v>
       </c>
       <c r="F17" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>pdfs/Inter-Faculty Cricket (2022).pdf</v>
       </c>
       <c r="G17" t="s">
-        <v>280</v>
+        <v>293</v>
       </c>
       <c r="I17" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.35">
@@ -3822,24 +3837,24 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>281</v>
+        <v>294</v>
       </c>
       <c r="C18" t="s">
-        <v>266</v>
+        <v>279</v>
       </c>
       <c r="E18" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>thumbs/Inter-Faculty Cricket (2023).webp</v>
       </c>
       <c r="F18" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>pdfs/Inter-Faculty Cricket (2023).pdf</v>
       </c>
       <c r="G18" t="s">
-        <v>280</v>
+        <v>293</v>
       </c>
       <c r="I18" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.35">
@@ -3847,24 +3862,24 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
       <c r="C19" t="s">
-        <v>266</v>
+        <v>279</v>
       </c>
       <c r="E19" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>thumbs/Leadership Program (2020).webp</v>
       </c>
       <c r="F19" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>pdfs/Leadership Program (2020).pdf</v>
       </c>
       <c r="G19" t="s">
-        <v>283</v>
+        <v>296</v>
       </c>
       <c r="I19" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.35">
@@ -3872,24 +3887,24 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>284</v>
+        <v>297</v>
       </c>
       <c r="C20" t="s">
-        <v>266</v>
+        <v>279</v>
       </c>
       <c r="E20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>thumbs/Leadership Program (2017).webp</v>
       </c>
       <c r="F20" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>pdfs/Leadership Program (2017).pdf</v>
       </c>
       <c r="G20" t="s">
-        <v>283</v>
+        <v>296</v>
       </c>
       <c r="I20" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.35">
@@ -3897,30 +3912,30 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>285</v>
+        <v>298</v>
       </c>
       <c r="C21" t="s">
-        <v>286</v>
+        <v>299</v>
       </c>
       <c r="D21" t="s">
-        <v>287</v>
+        <v>300</v>
       </c>
       <c r="E21" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>thumbs/Foundations of Project Management.webp</v>
       </c>
       <c r="F21" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>pdfs/Foundations of Project Management.pdf</v>
       </c>
       <c r="G21" t="s">
-        <v>283</v>
+        <v>296</v>
       </c>
       <c r="H21" t="s">
-        <v>288</v>
+        <v>301</v>
       </c>
       <c r="I21" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.35">
@@ -3928,30 +3943,30 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>289</v>
+        <v>302</v>
       </c>
       <c r="C22" t="s">
-        <v>286</v>
+        <v>299</v>
       </c>
       <c r="D22" t="s">
-        <v>290</v>
+        <v>303</v>
       </c>
       <c r="E22" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>thumbs/Project Initiation - Starting a Successful Project.webp</v>
       </c>
       <c r="F22" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>pdfs/Project Initiation - Starting a Successful Project.pdf</v>
       </c>
       <c r="G22" t="s">
-        <v>283</v>
+        <v>296</v>
       </c>
       <c r="H22" t="s">
-        <v>288</v>
+        <v>301</v>
       </c>
       <c r="I22" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.35">
@@ -3959,30 +3974,30 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>291</v>
+        <v>304</v>
       </c>
       <c r="C23" t="s">
-        <v>286</v>
+        <v>299</v>
       </c>
       <c r="D23" t="s">
-        <v>292</v>
+        <v>305</v>
       </c>
       <c r="E23" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>thumbs/Project Planning - Putting It All Together.webp</v>
       </c>
       <c r="F23" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>pdfs/Project Planning - Putting It All Together.pdf</v>
       </c>
       <c r="G23" t="s">
-        <v>283</v>
+        <v>296</v>
       </c>
       <c r="H23" t="s">
-        <v>288</v>
+        <v>301</v>
       </c>
       <c r="I23" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.35">
@@ -3990,27 +4005,27 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>293</v>
+        <v>306</v>
       </c>
       <c r="C24" t="s">
-        <v>264</v>
+        <v>276</v>
       </c>
       <c r="D24" t="s">
-        <v>294</v>
+        <v>307</v>
       </c>
       <c r="E24" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>thumbs/Introduction to Marketing.webp</v>
       </c>
       <c r="F24" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>pdfs/Introduction to Marketing.pdf</v>
       </c>
       <c r="G24" t="s">
-        <v>278</v>
+        <v>291</v>
       </c>
       <c r="I24" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.35">
@@ -4018,24 +4033,24 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>295</v>
+        <v>308</v>
       </c>
       <c r="C25" t="s">
-        <v>286</v>
+        <v>299</v>
       </c>
       <c r="E25" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>thumbs/Fundamentals of Digital Marketing.webp</v>
       </c>
       <c r="F25" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>pdfs/Fundamentals of Digital Marketing.pdf</v>
       </c>
       <c r="G25" t="s">
-        <v>296</v>
+        <v>309</v>
       </c>
       <c r="I25" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.35">
@@ -4043,30 +4058,30 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>297</v>
+        <v>310</v>
       </c>
       <c r="C26" t="s">
-        <v>298</v>
+        <v>311</v>
       </c>
       <c r="D26" t="s">
-        <v>299</v>
+        <v>312</v>
       </c>
       <c r="E26" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>thumbs/Claude 101.webp</v>
       </c>
       <c r="F26" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>pdfs/Claude 101.pdf</v>
       </c>
       <c r="G26" t="s">
-        <v>300</v>
+        <v>313</v>
       </c>
       <c r="H26" t="s">
-        <v>301</v>
+        <v>314</v>
       </c>
       <c r="I26" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.35">
@@ -4074,30 +4089,30 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>302</v>
+        <v>315</v>
       </c>
       <c r="C27" t="s">
-        <v>298</v>
+        <v>311</v>
       </c>
       <c r="D27" t="s">
-        <v>303</v>
+        <v>316</v>
       </c>
       <c r="E27" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>thumbs/Claude Code 101.webp</v>
       </c>
       <c r="F27" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>pdfs/Claude Code 101.pdf</v>
       </c>
       <c r="G27" t="s">
-        <v>300</v>
+        <v>313</v>
       </c>
       <c r="H27" t="s">
-        <v>301</v>
+        <v>314</v>
       </c>
       <c r="I27" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.35">
@@ -4105,30 +4120,30 @@
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>304</v>
+        <v>317</v>
       </c>
       <c r="C28" t="s">
-        <v>298</v>
+        <v>311</v>
       </c>
       <c r="D28" t="s">
-        <v>305</v>
+        <v>318</v>
       </c>
       <c r="E28" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>thumbs/Claude Platform 101.webp</v>
       </c>
       <c r="F28" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>pdfs/Claude Platform 101.pdf</v>
       </c>
       <c r="G28" t="s">
-        <v>300</v>
+        <v>313</v>
       </c>
       <c r="H28" t="s">
-        <v>301</v>
+        <v>314</v>
       </c>
       <c r="I28" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.35">
@@ -4136,30 +4151,30 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>306</v>
+        <v>319</v>
       </c>
       <c r="C29" t="s">
-        <v>298</v>
+        <v>311</v>
       </c>
       <c r="D29" t="s">
-        <v>307</v>
+        <v>320</v>
       </c>
       <c r="E29" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>thumbs/Introduction to Claude Cowork.webp</v>
       </c>
       <c r="F29" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>pdfs/Introduction to Claude Cowork.pdf</v>
       </c>
       <c r="G29" t="s">
-        <v>300</v>
+        <v>313</v>
       </c>
       <c r="H29" t="s">
-        <v>301</v>
+        <v>314</v>
       </c>
       <c r="I29" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.35">
@@ -4167,30 +4182,30 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>308</v>
+        <v>321</v>
       </c>
       <c r="C30" t="s">
-        <v>298</v>
+        <v>311</v>
       </c>
       <c r="D30" t="s">
-        <v>309</v>
+        <v>322</v>
       </c>
       <c r="E30" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>thumbs/Claude Code in Action.webp</v>
       </c>
       <c r="F30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>pdfs/Claude Code in Action.pdf</v>
       </c>
       <c r="G30" t="s">
-        <v>300</v>
+        <v>313</v>
       </c>
       <c r="H30" t="s">
-        <v>301</v>
+        <v>314</v>
       </c>
       <c r="I30" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.35">
@@ -4198,30 +4213,30 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>310</v>
+        <v>323</v>
       </c>
       <c r="C31" t="s">
-        <v>298</v>
+        <v>311</v>
       </c>
       <c r="D31" t="s">
-        <v>311</v>
+        <v>324</v>
       </c>
       <c r="E31" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>thumbs/AI Fluency - Frameworks &amp; Foundations.webp</v>
       </c>
       <c r="F31" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>pdfs/AI Fluency - Frameworks &amp; Foundations.pdf</v>
       </c>
       <c r="G31" t="s">
-        <v>300</v>
+        <v>313</v>
       </c>
       <c r="H31" t="s">
-        <v>301</v>
+        <v>314</v>
       </c>
       <c r="I31" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.35">
@@ -4229,30 +4244,30 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>312</v>
+        <v>325</v>
       </c>
       <c r="C32" t="s">
-        <v>298</v>
+        <v>311</v>
       </c>
       <c r="D32" t="s">
+        <v>326</v>
+      </c>
+      <c r="E32" t="str">
+        <f t="shared" si="0"/>
+        <v>thumbs/Introduction to Model Context Protocol.webp</v>
+      </c>
+      <c r="F32" t="str">
+        <f t="shared" si="1"/>
+        <v>pdfs/Introduction to Model Context Protocol.pdf</v>
+      </c>
+      <c r="G32" t="s">
         <v>313</v>
       </c>
-      <c r="E32" t="str">
-        <f t="shared" si="2"/>
-        <v>thumbs/Introduction to Model Context Protocol.webp</v>
-      </c>
-      <c r="F32" t="str">
-        <f t="shared" si="3"/>
-        <v>pdfs/Introduction to Model Context Protocol.pdf</v>
-      </c>
-      <c r="G32" t="s">
-        <v>300</v>
-      </c>
       <c r="H32" t="s">
-        <v>301</v>
+        <v>314</v>
       </c>
       <c r="I32" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.35">
@@ -4260,30 +4275,30 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
+        <v>327</v>
+      </c>
+      <c r="C33" t="s">
+        <v>311</v>
+      </c>
+      <c r="D33" t="s">
+        <v>328</v>
+      </c>
+      <c r="E33" t="str">
+        <f t="shared" si="0"/>
+        <v>thumbs/Model Context Protocol - Advanced Topics.webp</v>
+      </c>
+      <c r="F33" t="str">
+        <f t="shared" si="1"/>
+        <v>pdfs/Model Context Protocol - Advanced Topics.pdf</v>
+      </c>
+      <c r="G33" t="s">
+        <v>313</v>
+      </c>
+      <c r="H33" t="s">
         <v>314</v>
       </c>
-      <c r="C33" t="s">
-        <v>298</v>
-      </c>
-      <c r="D33" t="s">
-        <v>315</v>
-      </c>
-      <c r="E33" t="str">
-        <f t="shared" si="2"/>
-        <v>thumbs/Model Context Protocol - Advanced Topics.webp</v>
-      </c>
-      <c r="F33" t="str">
-        <f t="shared" si="3"/>
-        <v>pdfs/Model Context Protocol - Advanced Topics.pdf</v>
-      </c>
-      <c r="G33" t="s">
-        <v>300</v>
-      </c>
-      <c r="H33" t="s">
-        <v>301</v>
-      </c>
       <c r="I33" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.35">
@@ -4291,30 +4306,30 @@
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>316</v>
+        <v>329</v>
       </c>
       <c r="C34" t="s">
-        <v>298</v>
+        <v>311</v>
       </c>
       <c r="D34" t="s">
-        <v>317</v>
+        <v>330</v>
       </c>
       <c r="E34" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" ref="E34:E52" si="2">"thumbs/" &amp; B34 &amp; ".webp"</f>
         <v>thumbs/AI Fluency for Educators.webp</v>
       </c>
       <c r="F34" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" ref="F34:F52" si="3">"pdfs/" &amp; B34 &amp; ".pdf"</f>
         <v>pdfs/AI Fluency for Educators.pdf</v>
       </c>
       <c r="G34" t="s">
-        <v>300</v>
+        <v>313</v>
       </c>
       <c r="H34" t="s">
-        <v>301</v>
+        <v>314</v>
       </c>
       <c r="I34" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.35">
@@ -4322,13 +4337,13 @@
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>318</v>
+        <v>331</v>
       </c>
       <c r="C35" t="s">
-        <v>298</v>
+        <v>311</v>
       </c>
       <c r="D35" t="s">
-        <v>319</v>
+        <v>332</v>
       </c>
       <c r="E35" t="str">
         <f t="shared" si="2"/>
@@ -4339,13 +4354,13 @@
         <v>pdfs/AI Fluency for Students.pdf</v>
       </c>
       <c r="G35" t="s">
-        <v>300</v>
+        <v>313</v>
       </c>
       <c r="H35" t="s">
-        <v>301</v>
+        <v>314</v>
       </c>
       <c r="I35" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.35">
@@ -4353,13 +4368,13 @@
         <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>320</v>
+        <v>333</v>
       </c>
       <c r="C36" t="s">
-        <v>298</v>
+        <v>311</v>
       </c>
       <c r="D36" t="s">
-        <v>321</v>
+        <v>334</v>
       </c>
       <c r="E36" t="str">
         <f t="shared" si="2"/>
@@ -4370,13 +4385,13 @@
         <v>pdfs/Teaching the AI Fluency Framework.pdf</v>
       </c>
       <c r="G36" t="s">
-        <v>300</v>
+        <v>313</v>
       </c>
       <c r="H36" t="s">
-        <v>301</v>
+        <v>314</v>
       </c>
       <c r="I36" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.35">
@@ -4384,13 +4399,13 @@
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>322</v>
+        <v>335</v>
       </c>
       <c r="C37" t="s">
-        <v>298</v>
+        <v>311</v>
       </c>
       <c r="D37" t="s">
-        <v>323</v>
+        <v>336</v>
       </c>
       <c r="E37" t="str">
         <f t="shared" si="2"/>
@@ -4401,13 +4416,13 @@
         <v>pdfs/AI Fluency for Non-Profits.pdf</v>
       </c>
       <c r="G37" t="s">
-        <v>300</v>
+        <v>313</v>
       </c>
       <c r="H37" t="s">
-        <v>301</v>
+        <v>314</v>
       </c>
       <c r="I37" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.35">
@@ -4415,13 +4430,13 @@
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>324</v>
+        <v>337</v>
       </c>
       <c r="C38" t="s">
-        <v>298</v>
+        <v>311</v>
       </c>
       <c r="D38" t="s">
-        <v>325</v>
+        <v>338</v>
       </c>
       <c r="E38" t="str">
         <f t="shared" si="2"/>
@@ -4432,13 +4447,13 @@
         <v>pdfs/AI Fluency for Small Businesses.pdf</v>
       </c>
       <c r="G38" t="s">
-        <v>300</v>
+        <v>313</v>
       </c>
       <c r="H38" t="s">
-        <v>301</v>
+        <v>314</v>
       </c>
       <c r="I38" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.35">
@@ -4446,13 +4461,13 @@
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>326</v>
+        <v>339</v>
       </c>
       <c r="C39" t="s">
-        <v>298</v>
+        <v>311</v>
       </c>
       <c r="D39" t="s">
-        <v>327</v>
+        <v>340</v>
       </c>
       <c r="E39" t="str">
         <f t="shared" si="2"/>
@@ -4463,13 +4478,13 @@
         <v>pdfs/Introduction to Agent Skills.pdf</v>
       </c>
       <c r="G39" t="s">
-        <v>300</v>
+        <v>313</v>
       </c>
       <c r="H39" t="s">
-        <v>301</v>
+        <v>314</v>
       </c>
       <c r="I39" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.35">
@@ -4477,13 +4492,13 @@
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>328</v>
+        <v>341</v>
       </c>
       <c r="C40" t="s">
-        <v>298</v>
+        <v>311</v>
       </c>
       <c r="D40" t="s">
-        <v>329</v>
+        <v>342</v>
       </c>
       <c r="E40" t="str">
         <f t="shared" si="2"/>
@@ -4494,13 +4509,13 @@
         <v>pdfs/Introduction to Sub-Agents.pdf</v>
       </c>
       <c r="G40" t="s">
-        <v>300</v>
+        <v>313</v>
       </c>
       <c r="H40" t="s">
-        <v>301</v>
+        <v>314</v>
       </c>
       <c r="I40" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.35">
@@ -4508,13 +4523,13 @@
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>330</v>
+        <v>343</v>
       </c>
       <c r="C41" t="s">
-        <v>298</v>
+        <v>311</v>
       </c>
       <c r="D41" t="s">
-        <v>331</v>
+        <v>344</v>
       </c>
       <c r="E41" t="str">
         <f t="shared" si="2"/>
@@ -4525,13 +4540,13 @@
         <v>pdfs/AI Capabilities &amp; Limitations.pdf</v>
       </c>
       <c r="G41" t="s">
-        <v>300</v>
+        <v>313</v>
       </c>
       <c r="H41" t="s">
-        <v>301</v>
+        <v>314</v>
       </c>
       <c r="I41" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.35">
@@ -4539,13 +4554,13 @@
         <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>332</v>
+        <v>345</v>
       </c>
       <c r="C42" t="s">
-        <v>298</v>
+        <v>311</v>
       </c>
       <c r="D42" t="s">
-        <v>333</v>
+        <v>346</v>
       </c>
       <c r="E42" t="str">
         <f t="shared" si="2"/>
@@ -4556,13 +4571,13 @@
         <v>pdfs/Claude with Anthropic API.pdf</v>
       </c>
       <c r="G42" t="s">
-        <v>300</v>
+        <v>313</v>
       </c>
       <c r="H42" t="s">
-        <v>301</v>
+        <v>314</v>
       </c>
       <c r="I42" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.35">
@@ -4570,13 +4585,13 @@
         <v>42</v>
       </c>
       <c r="B43" t="s">
-        <v>334</v>
+        <v>347</v>
       </c>
       <c r="C43" t="s">
-        <v>298</v>
+        <v>311</v>
       </c>
       <c r="D43" t="s">
-        <v>335</v>
+        <v>348</v>
       </c>
       <c r="E43" t="str">
         <f t="shared" si="2"/>
@@ -4587,13 +4602,13 @@
         <v>pdfs/Claude with Google Vertex AI.pdf</v>
       </c>
       <c r="G43" t="s">
-        <v>300</v>
+        <v>313</v>
       </c>
       <c r="H43" t="s">
-        <v>301</v>
+        <v>314</v>
       </c>
       <c r="I43" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.35">
@@ -4601,13 +4616,13 @@
         <v>43</v>
       </c>
       <c r="B44" t="s">
-        <v>336</v>
+        <v>349</v>
       </c>
       <c r="C44" t="s">
-        <v>298</v>
+        <v>311</v>
       </c>
       <c r="D44" t="s">
-        <v>337</v>
+        <v>350</v>
       </c>
       <c r="E44" t="str">
         <f t="shared" si="2"/>
@@ -4618,13 +4633,13 @@
         <v>pdfs/Claude with Amazon Bedrock.pdf</v>
       </c>
       <c r="G44" t="s">
-        <v>300</v>
+        <v>313</v>
       </c>
       <c r="H44" t="s">
-        <v>301</v>
+        <v>314</v>
       </c>
       <c r="I44" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.35">
@@ -4632,13 +4647,13 @@
         <v>44</v>
       </c>
       <c r="B45" t="s">
-        <v>338</v>
+        <v>351</v>
       </c>
       <c r="C45" t="s">
-        <v>339</v>
+        <v>352</v>
       </c>
       <c r="D45" t="s">
-        <v>340</v>
+        <v>353</v>
       </c>
       <c r="E45" t="str">
         <f t="shared" si="2"/>
@@ -4649,10 +4664,10 @@
         <v>pdfs/Getting Started with Python.pdf</v>
       </c>
       <c r="G45" t="s">
-        <v>341</v>
+        <v>354</v>
       </c>
       <c r="I45" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.35">
@@ -4660,10 +4675,10 @@
         <v>45</v>
       </c>
       <c r="B46" t="s">
-        <v>342</v>
+        <v>355</v>
       </c>
       <c r="C46" t="s">
-        <v>343</v>
+        <v>356</v>
       </c>
       <c r="E46" t="str">
         <f t="shared" si="2"/>
@@ -4674,10 +4689,10 @@
         <v>pdfs/Gampaha District Cricket Team.pdf</v>
       </c>
       <c r="G46" t="s">
-        <v>280</v>
+        <v>293</v>
       </c>
       <c r="I46" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.35">
@@ -4685,10 +4700,10 @@
         <v>46</v>
       </c>
       <c r="B47" t="s">
-        <v>344</v>
+        <v>357</v>
       </c>
       <c r="C47" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="E47" t="str">
         <f t="shared" si="2"/>
@@ -4699,10 +4714,10 @@
         <v>pdfs/Sports Colors - Cricket.pdf</v>
       </c>
       <c r="G47" t="s">
-        <v>280</v>
+        <v>293</v>
       </c>
       <c r="I47" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.35">
@@ -4710,10 +4725,10 @@
         <v>47</v>
       </c>
       <c r="B48" t="s">
-        <v>345</v>
+        <v>358</v>
       </c>
       <c r="C48" t="s">
-        <v>346</v>
+        <v>359</v>
       </c>
       <c r="E48" t="str">
         <f t="shared" si="2"/>
@@ -4724,10 +4739,10 @@
         <v>pdfs/All-Island U19 DIII Semi-Finalists (2019).pdf</v>
       </c>
       <c r="G48" t="s">
-        <v>280</v>
+        <v>293</v>
       </c>
       <c r="I48" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.35">
@@ -4735,10 +4750,10 @@
         <v>48</v>
       </c>
       <c r="B49" t="s">
-        <v>347</v>
+        <v>360</v>
       </c>
       <c r="C49" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="E49" t="str">
         <f t="shared" si="2"/>
@@ -4749,10 +4764,10 @@
         <v>pdfs/School Leaving Certificate.pdf</v>
       </c>
       <c r="G49" t="s">
-        <v>348</v>
+        <v>361</v>
       </c>
       <c r="I49" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.35">
@@ -4760,10 +4775,10 @@
         <v>49</v>
       </c>
       <c r="B50" t="s">
-        <v>349</v>
+        <v>362</v>
       </c>
       <c r="C50" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="E50" t="str">
         <f t="shared" si="2"/>
@@ -4774,10 +4789,10 @@
         <v>pdfs/Character Certificate.pdf</v>
       </c>
       <c r="G50" t="s">
-        <v>348</v>
+        <v>361</v>
       </c>
       <c r="I50" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.35">
@@ -4785,10 +4800,10 @@
         <v>50</v>
       </c>
       <c r="B51" t="s">
-        <v>350</v>
+        <v>363</v>
       </c>
       <c r="C51" t="s">
-        <v>351</v>
+        <v>364</v>
       </c>
       <c r="E51" t="str">
         <f t="shared" si="2"/>
@@ -4799,10 +4814,10 @@
         <v>pdfs/Advanced Level Results.pdf</v>
       </c>
       <c r="G51" t="s">
-        <v>348</v>
+        <v>361</v>
       </c>
       <c r="I51" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.35">
@@ -4810,10 +4825,10 @@
         <v>51</v>
       </c>
       <c r="B52" t="s">
-        <v>352</v>
+        <v>365</v>
       </c>
       <c r="C52" t="s">
-        <v>353</v>
+        <v>366</v>
       </c>
       <c r="E52" t="str">
         <f t="shared" si="2"/>
@@ -4824,10 +4839,10 @@
         <v>pdfs/IGCSE OL Results.pdf</v>
       </c>
       <c r="G52" t="s">
-        <v>348</v>
+        <v>361</v>
       </c>
       <c r="I52" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
     </row>
   </sheetData>
@@ -4837,7 +4852,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="2.81640625" bestFit="1" customWidth="1"/>
@@ -4848,19 +4863,19 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="C1" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="D1" t="s">
-        <v>211</v>
+        <v>217</v>
       </c>
       <c r="E1" t="s">
-        <v>354</v>
+        <v>367</v>
       </c>
       <c r="F1" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
       <c r="G1" t="s">
         <v>22</v>
@@ -4868,300 +4883,324 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="B2" t="s">
-        <v>355</v>
+        <v>422</v>
       </c>
       <c r="C2" t="s">
-        <v>356</v>
+        <v>421</v>
       </c>
       <c r="D2" t="s">
-        <v>357</v>
+        <v>368</v>
       </c>
       <c r="E2" t="s">
-        <v>358</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Aerospace, Entrepreneurship</t>
-        </is>
+        <v>369</v>
+      </c>
+      <c r="F2" t="s">
+        <v>222</v>
       </c>
       <c r="G2" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="B3" t="s">
-        <v>359</v>
+        <v>370</v>
       </c>
       <c r="C3" t="s">
-        <v>407</v>
+        <v>371</v>
       </c>
       <c r="D3" t="s">
-        <v>360</v>
+        <v>372</v>
       </c>
       <c r="E3" t="s">
-        <v>361</v>
+        <v>373</v>
       </c>
       <c r="F3" t="s">
-        <v>216</v>
+        <v>374</v>
       </c>
       <c r="G3" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="B4" t="s">
-        <v>362</v>
+        <v>423</v>
       </c>
       <c r="C4" t="s">
-        <v>406</v>
+        <v>375</v>
       </c>
       <c r="D4" t="s">
-        <v>363</v>
+        <v>376</v>
       </c>
       <c r="E4" t="s">
-        <v>364</v>
+        <v>377</v>
       </c>
       <c r="F4" t="s">
-        <v>216</v>
+        <v>222</v>
       </c>
       <c r="G4" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="B5" t="s">
-        <v>365</v>
+        <v>378</v>
       </c>
       <c r="C5" t="s">
-        <v>366</v>
+        <v>379</v>
       </c>
       <c r="D5" t="s">
-        <v>367</v>
+        <v>380</v>
       </c>
       <c r="E5" t="s">
-        <v>368</v>
+        <v>381</v>
       </c>
       <c r="F5" t="s">
-        <v>216</v>
+        <v>222</v>
       </c>
       <c r="G5" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>369</v>
+        <v>424</v>
       </c>
       <c r="C6" t="s">
-        <v>370</v>
+        <v>382</v>
       </c>
       <c r="D6" t="s">
-        <v>371</v>
+        <v>383</v>
       </c>
       <c r="E6" t="s">
-        <v>372</v>
+        <v>384</v>
       </c>
       <c r="F6" t="s">
-        <v>216</v>
+        <v>222</v>
       </c>
       <c r="G6" t="s">
-        <v>219</v>
+        <v>231</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="B7" t="s">
-        <v>373</v>
+        <v>385</v>
       </c>
       <c r="C7" t="s">
-        <v>374</v>
+        <v>386</v>
       </c>
       <c r="D7" t="s">
-        <v>375</v>
+        <v>387</v>
       </c>
       <c r="E7" t="s">
-        <v>376</v>
+        <v>388</v>
       </c>
       <c r="F7" t="s">
-        <v>216</v>
+        <v>222</v>
       </c>
       <c r="G7" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B8" t="s">
-        <v>400</v>
+        <v>389</v>
       </c>
       <c r="C8" t="s">
-        <v>377</v>
+        <v>390</v>
       </c>
       <c r="D8" t="s">
-        <v>378</v>
+        <v>391</v>
       </c>
       <c r="E8" t="s">
-        <v>379</v>
+        <v>392</v>
       </c>
       <c r="F8" t="s">
-        <v>216</v>
+        <v>222</v>
       </c>
       <c r="G8" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>401</v>
+        <v>393</v>
       </c>
       <c r="C9" t="s">
-        <v>380</v>
+        <v>394</v>
       </c>
       <c r="D9" t="s">
-        <v>381</v>
+        <v>395</v>
       </c>
       <c r="E9" t="s">
-        <v>382</v>
+        <v>396</v>
       </c>
       <c r="F9" t="s">
-        <v>383</v>
+        <v>222</v>
       </c>
       <c r="G9" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="B10" t="s">
-        <v>384</v>
+        <v>397</v>
       </c>
       <c r="C10" t="s">
-        <v>385</v>
+        <v>398</v>
       </c>
       <c r="D10" t="s">
-        <v>386</v>
+        <v>399</v>
       </c>
       <c r="E10" t="s">
-        <v>387</v>
+        <v>400</v>
       </c>
       <c r="F10" t="s">
-        <v>280</v>
+        <v>251</v>
       </c>
       <c r="G10" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="B11" t="s">
-        <v>388</v>
+        <v>401</v>
       </c>
       <c r="C11" t="s">
-        <v>389</v>
+        <v>402</v>
       </c>
       <c r="D11" t="s">
-        <v>390</v>
+        <v>403</v>
       </c>
       <c r="E11" t="s">
-        <v>391</v>
+        <v>404</v>
       </c>
       <c r="F11" t="s">
-        <v>392</v>
+        <v>293</v>
       </c>
       <c r="G11" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="B12" t="s">
-        <v>402</v>
+        <v>405</v>
       </c>
       <c r="C12" t="s">
-        <v>393</v>
+        <v>406</v>
       </c>
       <c r="D12" t="s">
-        <v>394</v>
+        <v>407</v>
       </c>
       <c r="E12" t="s">
-        <v>395</v>
+        <v>408</v>
       </c>
       <c r="F12" t="s">
-        <v>280</v>
+        <v>409</v>
       </c>
       <c r="G12" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="B13" t="s">
-        <v>403</v>
+        <v>410</v>
       </c>
       <c r="C13" t="s">
-        <v>405</v>
+        <v>411</v>
       </c>
       <c r="D13" t="s">
-        <v>396</v>
+        <v>412</v>
       </c>
       <c r="E13" t="s">
-        <v>397</v>
+        <v>413</v>
       </c>
       <c r="F13" t="s">
-        <v>280</v>
+        <v>293</v>
       </c>
       <c r="G13" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="B14" t="s">
-        <v>398</v>
+        <v>414</v>
       </c>
       <c r="C14" t="s">
-        <v>404</v>
+        <v>415</v>
       </c>
       <c r="D14" t="s">
-        <v>399</v>
+        <v>416</v>
+      </c>
+      <c r="E14" t="s">
+        <v>417</v>
       </c>
       <c r="F14" t="s">
-        <v>280</v>
+        <v>293</v>
       </c>
       <c r="G14" t="s">
-        <v>219</v>
+        <v>225</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A15">
+        <v>1</v>
+      </c>
+      <c r="B15" t="s">
+        <v>418</v>
+      </c>
+      <c r="C15" t="s">
+        <v>419</v>
+      </c>
+      <c r="D15" t="s">
+        <v>420</v>
+      </c>
+      <c r="E15" t="s">
+        <v>369</v>
+      </c>
+      <c r="F15" t="s">
+        <v>293</v>
+      </c>
+      <c r="G15" t="s">
+        <v>225</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Rework Accolades landscape into a coherent alien dune-scape
</commit_message>
<xml_diff>
--- a/fetch.xlsx
+++ b/fetch.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ghz\Documents\Claude\Projects\000 Online Portfolio - vcperera\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2C4F7C6-A520-4B75-8B72-F844651C5924}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A366B67C-750F-429B-9F63-45D533248399}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="personas" sheetId="1" r:id="rId1"/>
@@ -3272,7 +3272,7 @@
         <v>240</v>
       </c>
       <c r="G5" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="H5" t="s">
         <v>231</v>

</xml_diff>

<commit_message>
Optimize images (~7MB lighter grids); fix Project 8 to WebP; smooth avatar scroll; document changes in README
</commit_message>
<xml_diff>
--- a/fetch.xlsx
+++ b/fetch.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ghz\Documents\Claude\Projects\000 Online Portfolio - vcperera\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A366B67C-750F-429B-9F63-45D533248399}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAAF3796-65EB-465C-8918-E8DA6A67B567}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="personas" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="751" uniqueCount="425">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="757" uniqueCount="429">
   <si>
     <t>ID</t>
   </si>
@@ -705,30 +705,613 @@
   </si>
   <si>
     <t>Winner: EIIS x Airbus Annual Space Entrepreneurship Challenge Solving the Space Debris Challenge in an Sustainable Manner</t>
+  </si>
+  <si>
+    <t>Aerospace</t>
+  </si>
+  <si>
+    <t>Project 7/7-1.webp</t>
+  </si>
+  <si>
+    <t>Project 7/7-1.webp|Project 7/7-2.webp|Project 7/7-3.webp|Project 7/7-4.webp</t>
+  </si>
+  <si>
+    <t>NO</t>
+  </si>
+  <si>
+    <t>Aerodynamics of a Nano-Coated Flat Plate</t>
+  </si>
+  <si>
+    <t>Numeric Approach (CFD) | Winner: Best Poster Presentation, 16th International Research Conference (IRC)</t>
+  </si>
+  <si>
+    <t>Project 6/6-1.webp</t>
+  </si>
+  <si>
+    <t>Project 6/6-1.webp|Project 6/6-2.webp|Project 6/6-3.webp|Project 6/6-4.webp|Project 6/6-5.webp|Project 6/6-6.webp|Project 6/6-7.webp|Project 6/6-8.webp</t>
+  </si>
+  <si>
+    <t>YES</t>
+  </si>
+  <si>
+    <t>Numeric Approach (CFD) | Winner: Best Research Project (2024), Department of Aeronautical Engineering</t>
+  </si>
+  <si>
+    <t>Project 5/5-1.webp</t>
+  </si>
+  <si>
+    <t>Project 5/5-1.webp|Project 5/5-2.webp|Project 5/5-3.webp|Project 5/5-4.webp|Project 5/5-5.webp</t>
+  </si>
+  <si>
+    <t>Experimental Approach (Lab) | Grant of LKR 1Mn Approved by Combinatorial Advanced Research &amp; Education (KDU-CARE)</t>
+  </si>
+  <si>
+    <t>Project 4/4-1.webp</t>
+  </si>
+  <si>
+    <t>Developing a 3D Model of a Jet Engine</t>
+  </si>
+  <si>
+    <t>Designing a Jet Engine from scratch using a 2D Draft as a Sketch Picture</t>
+  </si>
+  <si>
+    <t>Project 3/3-1.webp</t>
+  </si>
+  <si>
+    <t>Project 3/3-1.webp|Project 3/3-2.webp</t>
+  </si>
+  <si>
+    <t>Developing a 3D Model of an A380</t>
+  </si>
+  <si>
+    <t>Designing an A380 exterior from scratch using a 2D Draft as a Sketch Picture</t>
+  </si>
+  <si>
+    <t>Project 2/2-1.webp</t>
+  </si>
+  <si>
+    <t>HYDRATech: Local Nanocoating Production</t>
+  </si>
+  <si>
+    <t>1,300+ Applicants at Entry to Semi-Finalists:
+IEEE Innovation Nation Sri Lanka (2021)</t>
+  </si>
+  <si>
+    <t>Entrepreneurship</t>
+  </si>
+  <si>
+    <t>Project 1/1-1.webp</t>
+  </si>
+  <si>
+    <t>Project 1/1-1.webp|Project 1/1-2.webp|Project 1/1-3.webp</t>
+  </si>
+  <si>
+    <t>Issuer</t>
+  </si>
+  <si>
+    <t>Verification Link</t>
+  </si>
+  <si>
+    <t>Certificate</t>
+  </si>
+  <si>
+    <t>Subject</t>
+  </si>
+  <si>
+    <t>Series</t>
+  </si>
+  <si>
+    <t>Master of Arts - Space Entrepreneurship</t>
+  </si>
+  <si>
+    <t>EIIS</t>
+  </si>
+  <si>
+    <t>Aerospace Engineering, Business &amp; Entrepreneurship</t>
+  </si>
+  <si>
+    <t>Acceptance Letter - EIIS</t>
+  </si>
+  <si>
+    <t>Digitalisation in Aeronautics</t>
+  </si>
+  <si>
+    <t>Technical University of Munich</t>
+  </si>
+  <si>
+    <t>https://www.coursera.org/account/accomplishments/verify/3WUDH2EMK2LJ</t>
+  </si>
+  <si>
+    <t>Aerospace Engineering</t>
+  </si>
+  <si>
+    <t>TUM Digitalisation in Aerospace</t>
+  </si>
+  <si>
+    <t>Digitalisation in Space Research</t>
+  </si>
+  <si>
+    <t>https://www.coursera.org/account/accomplishments/verify/4E6HK8QDWH6H</t>
+  </si>
+  <si>
+    <t>Digitalisation in the Aerospace Industry</t>
+  </si>
+  <si>
+    <t>https://www.coursera.org/account/accomplishments/verify/L8PEPDQR6EKL</t>
+  </si>
+  <si>
+    <t>Aerospace Materials</t>
+  </si>
+  <si>
+    <t>Tomsk Aerospace University</t>
+  </si>
+  <si>
+    <t>https://www.coursera.org/account/accomplishments/verify/MBQSVGN6GVH9</t>
+  </si>
+  <si>
+    <t>Robotics - Aerial Robotics</t>
+  </si>
+  <si>
+    <t>University of Pennsylvania</t>
+  </si>
+  <si>
+    <t>https://www.coursera.org/account/accomplishments/verify/2NZXDQTQWSA7</t>
+  </si>
+  <si>
+    <t>Best Research Project</t>
+  </si>
+  <si>
+    <t>Kotelawala Defense University</t>
+  </si>
+  <si>
+    <t>Best Poster Presentation</t>
+  </si>
+  <si>
+    <t>KDU International Research Conference</t>
+  </si>
+  <si>
+    <t>Paper Presentation at IRC</t>
+  </si>
+  <si>
+    <t>BSc. (Hons) Aeronautical Engineering</t>
+  </si>
+  <si>
+    <t>SEDS</t>
+  </si>
+  <si>
+    <t>Chairperson - SEDS SL</t>
+  </si>
+  <si>
+    <t>President - SEDS KDU</t>
+  </si>
+  <si>
+    <t>Service Letter</t>
+  </si>
+  <si>
+    <t>Semi-Finalists - IEEE INSL 2021</t>
+  </si>
+  <si>
+    <t>IEEE INSL</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/feed/update/urn:li:activity:6856230081409499136/</t>
+  </si>
+  <si>
+    <t>Business &amp; Entrepreneurship</t>
+  </si>
+  <si>
+    <t>Inter-Faculty Cricket (2022)</t>
+  </si>
+  <si>
+    <t>Sports</t>
+  </si>
+  <si>
+    <t>Inter-Faculty Cricket (2023)</t>
+  </si>
+  <si>
+    <t>Leadership Program (2020)</t>
+  </si>
+  <si>
+    <t>Leadership &amp; Management</t>
+  </si>
+  <si>
+    <t>Leadership Program (2017)</t>
+  </si>
+  <si>
+    <t>Foundations of Project Management</t>
+  </si>
+  <si>
+    <t>Google</t>
+  </si>
+  <si>
+    <t>https://coursera.org/verify/ZXNFNKQYSMK3</t>
+  </si>
+  <si>
+    <t>Google Project Management</t>
+  </si>
+  <si>
+    <t>Project Initiation - Starting a Successful Project</t>
+  </si>
+  <si>
+    <t>https://coursera.org/verify/BJZGG598RWS8</t>
+  </si>
+  <si>
+    <t>Project Planning - Putting It All Together</t>
+  </si>
+  <si>
+    <t>https://coursera.org/verify/HCMMZJJPRT68</t>
+  </si>
+  <si>
+    <t>Introduction to Marketing</t>
+  </si>
+  <si>
+    <t>https://www.coursera.org/account/accomplishments/verify/N9ELLGLJ5JSS</t>
+  </si>
+  <si>
+    <t>Fundamentals of Digital Marketing</t>
+  </si>
+  <si>
+    <t>Digital Marketing</t>
+  </si>
+  <si>
+    <t>Claude 101</t>
+  </si>
+  <si>
+    <t>Anthropic</t>
+  </si>
+  <si>
+    <t>https://verify.skilljar.com/c/kvp3s5ir6n2t</t>
+  </si>
+  <si>
+    <t>Artificial Intelligence</t>
+  </si>
+  <si>
+    <t>Anthropic AI Curriculum</t>
+  </si>
+  <si>
+    <t>Claude Code 101</t>
+  </si>
+  <si>
+    <t>https://verify.skilljar.com/c/abbvrauishf5</t>
+  </si>
+  <si>
+    <t>Claude Platform 101</t>
+  </si>
+  <si>
+    <t>https://verify.skilljar.com/c/9iiahw7qfgku</t>
+  </si>
+  <si>
+    <t>Introduction to Claude Cowork</t>
+  </si>
+  <si>
+    <t>https://verify.skilljar.com/c/ksw8mdothntb</t>
+  </si>
+  <si>
+    <t>Claude Code in Action</t>
+  </si>
+  <si>
+    <t>https://verify.skilljar.com/c/zjtnrq3jsj37</t>
+  </si>
+  <si>
+    <t>AI Fluency - Frameworks &amp; Foundations</t>
+  </si>
+  <si>
+    <t>https://verify.skilljar.com/c/ziji9iknr4rs</t>
+  </si>
+  <si>
+    <t>Introduction to Model Context Protocol</t>
+  </si>
+  <si>
+    <t>https://verify.skilljar.com/c/8q3dx4s43rnb</t>
+  </si>
+  <si>
+    <t>Model Context Protocol - Advanced Topics</t>
+  </si>
+  <si>
+    <t>https://verify.skilljar.com/c/vxo27r2hm3c5</t>
+  </si>
+  <si>
+    <t>AI Fluency for Educators</t>
+  </si>
+  <si>
+    <t>https://verify.skilljar.com/c/nkudubifd9k9</t>
+  </si>
+  <si>
+    <t>AI Fluency for Students</t>
+  </si>
+  <si>
+    <t>https://verify.skilljar.com/c/opmc82urpi9r</t>
+  </si>
+  <si>
+    <t>Teaching the AI Fluency Framework</t>
+  </si>
+  <si>
+    <t>https://verify.skilljar.com/c/z4dhmjvqjgs9</t>
+  </si>
+  <si>
+    <t>AI Fluency for Non-Profits</t>
+  </si>
+  <si>
+    <t>https://verify.skilljar.com/c/63p6ibyg359x</t>
+  </si>
+  <si>
+    <t>AI Fluency for Small Businesses</t>
+  </si>
+  <si>
+    <t>https://verify.skilljar.com/c/ogn6rbwcgspk</t>
+  </si>
+  <si>
+    <t>Introduction to Agent Skills</t>
+  </si>
+  <si>
+    <t>https://verify.skilljar.com/c/7fgvgpbe3748</t>
+  </si>
+  <si>
+    <t>Introduction to Sub-Agents</t>
+  </si>
+  <si>
+    <t>https://verify.skilljar.com/c/ud8upnkzvaw5</t>
+  </si>
+  <si>
+    <t>AI Capabilities &amp; Limitations</t>
+  </si>
+  <si>
+    <t>https://verify.skilljar.com/c/jbzi5nvbu8mq</t>
+  </si>
+  <si>
+    <t>Claude with Anthropic API</t>
+  </si>
+  <si>
+    <t>https://verify.skilljar.com/c/k3cc8hxpsnrz</t>
+  </si>
+  <si>
+    <t>Claude with Google Vertex AI</t>
+  </si>
+  <si>
+    <t>https://verify.skilljar.com/c/2hfhvkfsyo6x</t>
+  </si>
+  <si>
+    <t>Claude with Amazon Bedrock</t>
+  </si>
+  <si>
+    <t>https://verify.skilljar.com/c/8s2ai6kfaduc</t>
+  </si>
+  <si>
+    <t>Getting Started with Python</t>
+  </si>
+  <si>
+    <t>University of Michigan</t>
+  </si>
+  <si>
+    <t>https://www.coursera.org/account/accomplishments/verify/2XHJWDZB2XSY</t>
+  </si>
+  <si>
+    <t>Programming &amp; IT</t>
+  </si>
+  <si>
+    <t>Gampaha District Cricket Team</t>
+  </si>
+  <si>
+    <t>GDCA &amp; Sri Lanka Cricket</t>
+  </si>
+  <si>
+    <t>Sports Colors - Cricket</t>
+  </si>
+  <si>
+    <t>All-Island U19 DIII Semi-Finalists (2019)</t>
+  </si>
+  <si>
+    <t>Sri Lanka Schools Cricket Association</t>
+  </si>
+  <si>
+    <t>School Leaving Certificate</t>
+  </si>
+  <si>
+    <t>School</t>
+  </si>
+  <si>
+    <t>Character Certificate</t>
+  </si>
+  <si>
+    <t>Advanced Level Results</t>
+  </si>
+  <si>
+    <t>Department of Examintaions SL</t>
+  </si>
+  <si>
+    <t>IGCSE OL Results</t>
+  </si>
+  <si>
+    <t>Cambridge International Examinations</t>
+  </si>
+  <si>
+    <t>Post_Link</t>
+  </si>
+  <si>
+    <t>thumbs/14.webp</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/posts/the-futures-forum_spaceungana2026-spacefuturesforum-nextgenleaders-activity-7484926325519134720-dpOL?utm_source=share&amp;utm_medium=member_desktop&amp;rcm=ACoAADSwLqIBLzQLDm-Klx9wMM6NKZChtEvLQUo</t>
+  </si>
+  <si>
+    <t>Winners: Space Entrepreneurship Challenge</t>
+  </si>
+  <si>
+    <t>5th Edition organized by EIIS with Airbus D&amp;S, tied to the Master of Arts in Space Entrepreneurship.</t>
+  </si>
+  <si>
+    <t>thumbs/13.webp</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/posts/melodi-askelof_innovation-resilience-execution-activity-7460594246371434496-iSyu?utm_source=share&amp;utm_medium=member_desktop&amp;rcm=ACoAADSwLqIBLzQLDm-Klx9wMM6NKZChtEvLQUo</t>
+  </si>
+  <si>
+    <t>Aerospace, Entrepreneurship</t>
+  </si>
+  <si>
+    <t>Recognised as the Best Overall Local Chapter by SEDS Sri Lanka, within two years of its inception.</t>
+  </si>
+  <si>
+    <t>thumbs/12.webp</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/posts/seds-kdu_sedskdu-bestoverallchapter-teamwork-activity-7315058728968286208-UoCm?utm_source=social_share_send&amp;utm_medium=android_app&amp;rcm=ACoAADSwLqIBLzQLDm-Klx9wMM6NKZChtEvLQUo&amp;utm_campaign=copy_link</t>
+  </si>
+  <si>
+    <t>Vishal Appointed as Chairperson of SEDS SL</t>
+  </si>
+  <si>
+    <t>Leading the 7th Board of Directors and Board of Staff of SEDS Sri Lanka (2024/25).</t>
+  </si>
+  <si>
+    <t>thumbs/11.webp</t>
+  </si>
+  <si>
+    <t>https://foe.kdu.ac.lk/aero/2024/04/18/vishal-perera-appointed-as-chairperson-seds-sri-lanka-39</t>
+  </si>
+  <si>
+    <t>Awarded by the Department of Aeronautical Engineering at the Final Year Exhibition, KDU.</t>
+  </si>
+  <si>
+    <t>thumbs/10.webp</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/p/C4Vd0d1REmQ/?igsh=MWw1YTY1emcxcDM5Yg==</t>
+  </si>
+  <si>
+    <t>Congratulations: Vishal Perera of SEDS KDU!</t>
+  </si>
+  <si>
+    <t>Congratulatory post by SEDS KDU for the role ahead as National Chairperson.</t>
+  </si>
+  <si>
+    <t>thumbs/9.webp</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/p/C4Sr1ssxqcH/?igsh=MXVidWI1OTRlZG9pcQ==</t>
+  </si>
+  <si>
+    <t>Introducing the Chairperson of SEDS SL</t>
+  </si>
+  <si>
+    <t>Introductory Feature on the newly appointed Board of Directors of SEDS Sri Lanka, 2024-25.</t>
+  </si>
+  <si>
+    <t>thumbs/8.webp</t>
+  </si>
+  <si>
+    <t>https://foe.kdu.ac.lk/aero/2022/08/13/formation-of-the-space-force-27</t>
+  </si>
+  <si>
+    <t>Formation of the “Space Force”</t>
+  </si>
+  <si>
+    <t>Article on the formation of the SEDS KDU Local Chapter as the Founding Board.</t>
+  </si>
+  <si>
+    <t>thumbs/7.webp</t>
+  </si>
+  <si>
+    <t>https://foe.kdu.ac.lk/aero/2024/01/24/final-year-project-exhibition-2024-35</t>
+  </si>
+  <si>
+    <t>Semi Finalists: IEEE Innovation Nation SL</t>
+  </si>
+  <si>
+    <t>Conceptualizing a startup aiming to produce nanotech based coatings, locally.</t>
+  </si>
+  <si>
+    <t>thumbs/6.webp</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/IEEEINSL/posts/here-we-present-to-you-the-most-talented-semi-finalists-whose-hard-work-dedicati/3027737500833258/</t>
+  </si>
+  <si>
+    <t>Winners: Pentathlon 2022</t>
+  </si>
+  <si>
+    <t>An inter-university article-writing competition hosted by MoraSpirit, a premier sports network.</t>
+  </si>
+  <si>
+    <t>thumbs/5.webp</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/MoraSpirit/posts/after-a-close-competition-between-all-the-participants-we-are-pleased-to-inform-/424187246412243/</t>
+  </si>
+  <si>
+    <t>Climate Crisis and Clean Energy</t>
+  </si>
+  <si>
+    <t>Article on the Severity of the Climate Crisis. Competition organized by the IEEE SLTC.</t>
+  </si>
+  <si>
+    <t>thumbs/4.webp</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/photo?fbid=1106724503145581&amp;set=a.1106720086479356</t>
+  </si>
+  <si>
+    <t>Clean Energy</t>
+  </si>
+  <si>
+    <t>Top 8: Most Popular Schoolboy Cricketers</t>
+  </si>
+  <si>
+    <t>batsman.lk nominee based on performers at the All-Island School's Cricket Tournament (D2) 2019</t>
+  </si>
+  <si>
+    <t>thumbs/3.webp</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/reel/2660611044253733</t>
+  </si>
+  <si>
+    <t>Stats Alert: 176 Runs vs Royal Panadura</t>
+  </si>
+  <si>
+    <t>"Vishal Perera's 176 was the highlight for the Wattala boys in that game."</t>
+  </si>
+  <si>
+    <t>thumbs/2.webp</t>
+  </si>
+  <si>
+    <t>https://www.thepapare.com/u19-schools-cricket-division-2-1st-week-of-january-2020-roundup/</t>
+  </si>
+  <si>
+    <t>Daily News: 176 Runs vs Royal Panadura</t>
+  </si>
+  <si>
+    <t>"Vishal Perera skipper and right hand opener of LISW scored 176 runs in 202 balls…"</t>
+  </si>
+  <si>
+    <t>thumbs/1.webp</t>
+  </si>
+  <si>
+    <t>Africa's premier virtual forum on space futures, innovation and collaboration.</t>
+  </si>
+  <si>
+    <t>Distinguished Panelist: SPACE UNGANA '26</t>
+  </si>
+  <si>
+    <t>SEDS KDU: SEDS SL's Best Local Chapter</t>
+  </si>
+  <si>
+    <t>Best Research Project: Aero Engineering</t>
+  </si>
+  <si>
+    <t>Achieved Orbital: AeroLite</t>
+  </si>
+  <si>
+    <t>Aerodynamics of a Nano-Coated Airfoil #1</t>
+  </si>
+  <si>
+    <t>Aerodynamics of a Nano-Coated Airfoil #2</t>
   </si>
   <si>
     <t>As space based assets increase exponentially, so does the threat of Space Debris. The major problem is: who is going to pay to
 pick out the trash? Especially when it is flying past seven times the speed of a Sniper bullet in Low Earth Orbit. The Kessler
 Syndrome could lead to the immediate demise of the Space Economy. So whose to solve it and how?
 Aquila Aerospace set it's scope to directly tackle a regulatory requirements for Space Debris Mitigation: Passivation. Instead of "policing" space assets, we've conceptualized a novel network of onboard sensors and a SaaS such that it benefits operators, in-orbit services providers, regulators, insurers and SSA/STM service providers (TRL 2-3).</t>
-  </si>
-  <si>
-    <t>Aerospace</t>
-  </si>
-  <si>
-    <t>Project 7/7-1.webp</t>
-  </si>
-  <si>
-    <t>Project 7/7-1.webp|Project 7/7-2.webp|Project 7/7-3.webp|Project 7/7-4.webp</t>
-  </si>
-  <si>
-    <t>NO</t>
-  </si>
-  <si>
-    <t>Aerodynamics of a Nano-Coated Flat Plate</t>
-  </si>
-  <si>
-    <t>Numeric Approach (CFD) | Winner: Best Poster Presentation, 16th International Research Conference (IRC)</t>
   </si>
   <si>
     <t>Superhydrophobic Surfaces are cool. They are self-cleaning, anti-corrosive, anti-microbial, anti-icing and anti-biofouling
@@ -739,37 +1322,10 @@
 helped analyze what the most optimal degree of coating would be to achieve the best aerodynamics possible.</t>
   </si>
   <si>
-    <t>Project 6/6-1.webp</t>
-  </si>
-  <si>
-    <t>Project 6/6-1.webp|Project 6/6-2.webp|Project 6/6-3.webp|Project 6/6-4.webp|Project 6/6-5.webp|Project 6/6-6.webp|Project 6/6-7.webp|Project 6/6-8.webp</t>
-  </si>
-  <si>
-    <t>YES</t>
-  </si>
-  <si>
-    <t>Aerodynamics of a Nano-Coated Airfoil 1/2</t>
-  </si>
-  <si>
-    <t>Numeric Approach (CFD) | Winner: Best Research Project (2024), Department of Aeronautical Engineering</t>
-  </si>
-  <si>
     <t>Superhydrophobic Surfaces are still cool. In Project 1, the novel study discovered that the superhydrophobic surface properties had
 a positive impact on the overall aerodynamics of the flat plate and the relationship of aerodynamics with the coated area was non-linear. How would it fair with the aerodynamic body being an Airfoil? Would it have more exaggerated effects?
 In this secondary study I used OpenFOAM and SolidWorks to assess the aerodynamics of a NACA 4412 Airfoil, bearing the same principle
 mode of analysis as in Project #1, but for multiple Angles of Attack. Once again, superhydrophobic airfoils, especially those that are partially superhydrophobic, outperformed conventional uncoated airfoils and fully superhydrophobic airfoils.</t>
-  </si>
-  <si>
-    <t>Project 5/5-1.webp</t>
-  </si>
-  <si>
-    <t>Project 5/5-1.webp|Project 5/5-2.webp|Project 5/5-3.webp|Project 5/5-4.webp|Project 5/5-5.webp</t>
-  </si>
-  <si>
-    <t>Aerodynamics of a Nano-Coated Airfoil 2/2</t>
-  </si>
-  <si>
-    <t>Experimental Approach (Lab) | Grant of LKR 1Mn Approved by Combinatorial Advanced Research &amp; Education (KDU-CARE)</t>
   </si>
   <si>
     <t>Yes. Superhydrophobic surfaces are still cool as they were. Projects 1 and 2 had proved that there are positive benefits of
@@ -779,562 +1335,18 @@
 representatives of KDU-CARE. It was decided that a research grant of 1 Million LKR would be awarded, however, due to administrative delays, the project did not kickoff and was paused indefinitely.</t>
   </si>
   <si>
-    <t>Project 4/4-1.webp</t>
-  </si>
-  <si>
-    <t>Developing a 3D Model of a Jet Engine</t>
-  </si>
-  <si>
-    <t>Designing a Jet Engine from scratch using a 2D Draft as a Sketch Picture</t>
-  </si>
-  <si>
-    <t>Project 3/3-1.webp</t>
-  </si>
-  <si>
-    <t>Project 3/3-1.webp|Project 3/3-2.webp</t>
-  </si>
-  <si>
-    <t>Developing a 3D Model of an A380</t>
-  </si>
-  <si>
-    <t>Designing an A380 exterior from scratch using a 2D Draft as a Sketch Picture</t>
-  </si>
-  <si>
-    <t>Project 2/2-1.webp</t>
-  </si>
-  <si>
-    <t>HYDRATech: Local Nanocoating Production</t>
-  </si>
-  <si>
-    <t>1,300+ Applicants at Entry to Semi-Finalists:
-IEEE Innovation Nation Sri Lanka (2021)</t>
-  </si>
-  <si>
     <t>IEEE Innovation Nation Sri Lanka (INSL) is a premier national pre-accelerator program designed to cultivate an entrepreneurial and innovation-driven culture among young innovators and university students. Organized by the IEEE Sri Lanka Section, it empowers early-stage startups through intensive training, mentorship, and opportunities to secure seed funding and investor backing.
 HYDRATech aimed at manufacturing Superhydrophobic coatings in Sri Lanka, by prioritizing locally available resources. Superhydrophobic surfaces are inherently water-repellent surfaces due to the presence of unique nanostructures on the surface. The project failed
 to make it through to the final stage due to the Capital Intensive nature of the project.</t>
   </si>
   <si>
-    <t>Entrepreneurship</t>
-  </si>
-  <si>
-    <t>Project 1/1-1.webp</t>
-  </si>
-  <si>
-    <t>Project 1/1-1.webp|Project 1/1-2.webp|Project 1/1-3.webp</t>
-  </si>
-  <si>
-    <t>Issuer</t>
-  </si>
-  <si>
-    <t>Verification Link</t>
-  </si>
-  <si>
-    <t>Certificate</t>
-  </si>
-  <si>
-    <t>Subject</t>
-  </si>
-  <si>
-    <t>Series</t>
-  </si>
-  <si>
-    <t>Master of Arts - Space Entrepreneurship</t>
-  </si>
-  <si>
-    <t>EIIS</t>
-  </si>
-  <si>
-    <t>Aerospace Engineering, Business &amp; Entrepreneurship</t>
-  </si>
-  <si>
-    <t>Acceptance Letter - EIIS</t>
-  </si>
-  <si>
-    <t>Digitalisation in Aeronautics</t>
-  </si>
-  <si>
-    <t>Technical University of Munich</t>
-  </si>
-  <si>
-    <t>https://www.coursera.org/account/accomplishments/verify/3WUDH2EMK2LJ</t>
-  </si>
-  <si>
-    <t>Aerospace Engineering</t>
-  </si>
-  <si>
-    <t>TUM Digitalisation in Aerospace</t>
-  </si>
-  <si>
-    <t>Digitalisation in Space Research</t>
-  </si>
-  <si>
-    <t>https://www.coursera.org/account/accomplishments/verify/4E6HK8QDWH6H</t>
-  </si>
-  <si>
-    <t>Digitalisation in the Aerospace Industry</t>
-  </si>
-  <si>
-    <t>https://www.coursera.org/account/accomplishments/verify/L8PEPDQR6EKL</t>
-  </si>
-  <si>
-    <t>Aerospace Materials</t>
-  </si>
-  <si>
-    <t>Tomsk Aerospace University</t>
-  </si>
-  <si>
-    <t>https://www.coursera.org/account/accomplishments/verify/MBQSVGN6GVH9</t>
-  </si>
-  <si>
-    <t>Robotics - Aerial Robotics</t>
-  </si>
-  <si>
-    <t>University of Pennsylvania</t>
-  </si>
-  <si>
-    <t>https://www.coursera.org/account/accomplishments/verify/2NZXDQTQWSA7</t>
-  </si>
-  <si>
-    <t>Best Research Project</t>
-  </si>
-  <si>
-    <t>Kotelawala Defense University</t>
-  </si>
-  <si>
-    <t>Best Poster Presentation</t>
-  </si>
-  <si>
-    <t>KDU International Research Conference</t>
-  </si>
-  <si>
-    <t>Paper Presentation at IRC</t>
-  </si>
-  <si>
-    <t>BSc. (Hons) Aeronautical Engineering</t>
-  </si>
-  <si>
-    <t>SEDS</t>
-  </si>
-  <si>
-    <t>Chairperson - SEDS SL</t>
-  </si>
-  <si>
-    <t>President - SEDS KDU</t>
-  </si>
-  <si>
-    <t>Service Letter</t>
-  </si>
-  <si>
-    <t>Semi-Finalists - IEEE INSL 2021</t>
-  </si>
-  <si>
-    <t>IEEE INSL</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/feed/update/urn:li:activity:6856230081409499136/</t>
-  </si>
-  <si>
-    <t>Business &amp; Entrepreneurship</t>
-  </si>
-  <si>
-    <t>Inter-Faculty Cricket (2022)</t>
-  </si>
-  <si>
-    <t>Sports</t>
-  </si>
-  <si>
-    <t>Inter-Faculty Cricket (2023)</t>
-  </si>
-  <si>
-    <t>Leadership Program (2020)</t>
-  </si>
-  <si>
-    <t>Leadership &amp; Management</t>
-  </si>
-  <si>
-    <t>Leadership Program (2017)</t>
-  </si>
-  <si>
-    <t>Foundations of Project Management</t>
-  </si>
-  <si>
-    <t>Google</t>
-  </si>
-  <si>
-    <t>https://coursera.org/verify/ZXNFNKQYSMK3</t>
-  </si>
-  <si>
-    <t>Google Project Management</t>
-  </si>
-  <si>
-    <t>Project Initiation - Starting a Successful Project</t>
-  </si>
-  <si>
-    <t>https://coursera.org/verify/BJZGG598RWS8</t>
-  </si>
-  <si>
-    <t>Project Planning - Putting It All Together</t>
-  </si>
-  <si>
-    <t>https://coursera.org/verify/HCMMZJJPRT68</t>
-  </si>
-  <si>
-    <t>Introduction to Marketing</t>
-  </si>
-  <si>
-    <t>https://www.coursera.org/account/accomplishments/verify/N9ELLGLJ5JSS</t>
-  </si>
-  <si>
-    <t>Fundamentals of Digital Marketing</t>
-  </si>
-  <si>
-    <t>Digital Marketing</t>
-  </si>
-  <si>
-    <t>Claude 101</t>
-  </si>
-  <si>
-    <t>Anthropic</t>
-  </si>
-  <si>
-    <t>https://verify.skilljar.com/c/kvp3s5ir6n2t</t>
-  </si>
-  <si>
-    <t>Artificial Intelligence</t>
-  </si>
-  <si>
-    <t>Anthropic AI Curriculum</t>
-  </si>
-  <si>
-    <t>Claude Code 101</t>
-  </si>
-  <si>
-    <t>https://verify.skilljar.com/c/abbvrauishf5</t>
-  </si>
-  <si>
-    <t>Claude Platform 101</t>
-  </si>
-  <si>
-    <t>https://verify.skilljar.com/c/9iiahw7qfgku</t>
-  </si>
-  <si>
-    <t>Introduction to Claude Cowork</t>
-  </si>
-  <si>
-    <t>https://verify.skilljar.com/c/ksw8mdothntb</t>
-  </si>
-  <si>
-    <t>Claude Code in Action</t>
-  </si>
-  <si>
-    <t>https://verify.skilljar.com/c/zjtnrq3jsj37</t>
-  </si>
-  <si>
-    <t>AI Fluency - Frameworks &amp; Foundations</t>
-  </si>
-  <si>
-    <t>https://verify.skilljar.com/c/ziji9iknr4rs</t>
-  </si>
-  <si>
-    <t>Introduction to Model Context Protocol</t>
-  </si>
-  <si>
-    <t>https://verify.skilljar.com/c/8q3dx4s43rnb</t>
-  </si>
-  <si>
-    <t>Model Context Protocol - Advanced Topics</t>
-  </si>
-  <si>
-    <t>https://verify.skilljar.com/c/vxo27r2hm3c5</t>
-  </si>
-  <si>
-    <t>AI Fluency for Educators</t>
-  </si>
-  <si>
-    <t>https://verify.skilljar.com/c/nkudubifd9k9</t>
-  </si>
-  <si>
-    <t>AI Fluency for Students</t>
-  </si>
-  <si>
-    <t>https://verify.skilljar.com/c/opmc82urpi9r</t>
-  </si>
-  <si>
-    <t>Teaching the AI Fluency Framework</t>
-  </si>
-  <si>
-    <t>https://verify.skilljar.com/c/z4dhmjvqjgs9</t>
-  </si>
-  <si>
-    <t>AI Fluency for Non-Profits</t>
-  </si>
-  <si>
-    <t>https://verify.skilljar.com/c/63p6ibyg359x</t>
-  </si>
-  <si>
-    <t>AI Fluency for Small Businesses</t>
-  </si>
-  <si>
-    <t>https://verify.skilljar.com/c/ogn6rbwcgspk</t>
-  </si>
-  <si>
-    <t>Introduction to Agent Skills</t>
-  </si>
-  <si>
-    <t>https://verify.skilljar.com/c/7fgvgpbe3748</t>
-  </si>
-  <si>
-    <t>Introduction to Sub-Agents</t>
-  </si>
-  <si>
-    <t>https://verify.skilljar.com/c/ud8upnkzvaw5</t>
-  </si>
-  <si>
-    <t>AI Capabilities &amp; Limitations</t>
-  </si>
-  <si>
-    <t>https://verify.skilljar.com/c/jbzi5nvbu8mq</t>
-  </si>
-  <si>
-    <t>Claude with Anthropic API</t>
-  </si>
-  <si>
-    <t>https://verify.skilljar.com/c/k3cc8hxpsnrz</t>
-  </si>
-  <si>
-    <t>Claude with Google Vertex AI</t>
-  </si>
-  <si>
-    <t>https://verify.skilljar.com/c/2hfhvkfsyo6x</t>
-  </si>
-  <si>
-    <t>Claude with Amazon Bedrock</t>
-  </si>
-  <si>
-    <t>https://verify.skilljar.com/c/8s2ai6kfaduc</t>
-  </si>
-  <si>
-    <t>Getting Started with Python</t>
-  </si>
-  <si>
-    <t>University of Michigan</t>
-  </si>
-  <si>
-    <t>https://www.coursera.org/account/accomplishments/verify/2XHJWDZB2XSY</t>
-  </si>
-  <si>
-    <t>Programming &amp; IT</t>
-  </si>
-  <si>
-    <t>Gampaha District Cricket Team</t>
-  </si>
-  <si>
-    <t>GDCA &amp; Sri Lanka Cricket</t>
-  </si>
-  <si>
-    <t>Sports Colors - Cricket</t>
-  </si>
-  <si>
-    <t>All-Island U19 DIII Semi-Finalists (2019)</t>
-  </si>
-  <si>
-    <t>Sri Lanka Schools Cricket Association</t>
-  </si>
-  <si>
-    <t>School Leaving Certificate</t>
-  </si>
-  <si>
-    <t>School</t>
-  </si>
-  <si>
-    <t>Character Certificate</t>
-  </si>
-  <si>
-    <t>Advanced Level Results</t>
-  </si>
-  <si>
-    <t>Department of Examintaions SL</t>
-  </si>
-  <si>
-    <t>IGCSE OL Results</t>
-  </si>
-  <si>
-    <t>Cambridge International Examinations</t>
-  </si>
-  <si>
-    <t>Post_Link</t>
-  </si>
-  <si>
-    <t>thumbs/14.webp</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/posts/the-futures-forum_spaceungana2026-spacefuturesforum-nextgenleaders-activity-7484926325519134720-dpOL?utm_source=share&amp;utm_medium=member_desktop&amp;rcm=ACoAADSwLqIBLzQLDm-Klx9wMM6NKZChtEvLQUo</t>
-  </si>
-  <si>
-    <t>Winners: Space Entrepreneurship Challenge</t>
-  </si>
-  <si>
-    <t>5th Edition organized by EIIS with Airbus D&amp;S, tied to the Master of Arts in Space Entrepreneurship.</t>
-  </si>
-  <si>
-    <t>thumbs/13.webp</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/posts/melodi-askelof_innovation-resilience-execution-activity-7460594246371434496-iSyu?utm_source=share&amp;utm_medium=member_desktop&amp;rcm=ACoAADSwLqIBLzQLDm-Klx9wMM6NKZChtEvLQUo</t>
-  </si>
-  <si>
-    <t>Aerospace, Entrepreneurship</t>
-  </si>
-  <si>
-    <t>Recognised as the Best Overall Local Chapter by SEDS Sri Lanka, within two years of its inception.</t>
-  </si>
-  <si>
-    <t>thumbs/12.webp</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/posts/seds-kdu_sedskdu-bestoverallchapter-teamwork-activity-7315058728968286208-UoCm?utm_source=social_share_send&amp;utm_medium=android_app&amp;rcm=ACoAADSwLqIBLzQLDm-Klx9wMM6NKZChtEvLQUo&amp;utm_campaign=copy_link</t>
-  </si>
-  <si>
-    <t>Vishal Appointed as Chairperson of SEDS SL</t>
-  </si>
-  <si>
-    <t>Leading the 7th Board of Directors and Board of Staff of SEDS Sri Lanka (2024/25).</t>
-  </si>
-  <si>
-    <t>thumbs/11.webp</t>
-  </si>
-  <si>
-    <t>https://foe.kdu.ac.lk/aero/2024/04/18/vishal-perera-appointed-as-chairperson-seds-sri-lanka-39</t>
-  </si>
-  <si>
-    <t>Awarded by the Department of Aeronautical Engineering at the Final Year Exhibition, KDU.</t>
-  </si>
-  <si>
-    <t>thumbs/10.webp</t>
-  </si>
-  <si>
-    <t>https://www.instagram.com/p/C4Vd0d1REmQ/?igsh=MWw1YTY1emcxcDM5Yg==</t>
-  </si>
-  <si>
-    <t>Congratulations: Vishal Perera of SEDS KDU!</t>
-  </si>
-  <si>
-    <t>Congratulatory post by SEDS KDU for the role ahead as National Chairperson.</t>
-  </si>
-  <si>
-    <t>thumbs/9.webp</t>
-  </si>
-  <si>
-    <t>https://www.instagram.com/p/C4Sr1ssxqcH/?igsh=MXVidWI1OTRlZG9pcQ==</t>
-  </si>
-  <si>
-    <t>Introducing the Chairperson of SEDS SL</t>
-  </si>
-  <si>
-    <t>Introductory Feature on the newly appointed Board of Directors of SEDS Sri Lanka, 2024-25.</t>
-  </si>
-  <si>
-    <t>thumbs/8.webp</t>
-  </si>
-  <si>
-    <t>https://foe.kdu.ac.lk/aero/2022/08/13/formation-of-the-space-force-27</t>
-  </si>
-  <si>
-    <t>Formation of the “Space Force”</t>
-  </si>
-  <si>
-    <t>Article on the formation of the SEDS KDU Local Chapter as the Founding Board.</t>
-  </si>
-  <si>
-    <t>thumbs/7.webp</t>
-  </si>
-  <si>
-    <t>https://foe.kdu.ac.lk/aero/2024/01/24/final-year-project-exhibition-2024-35</t>
-  </si>
-  <si>
-    <t>Semi Finalists: IEEE Innovation Nation SL</t>
-  </si>
-  <si>
-    <t>Conceptualizing a startup aiming to produce nanotech based coatings, locally.</t>
-  </si>
-  <si>
-    <t>thumbs/6.webp</t>
-  </si>
-  <si>
-    <t>https://www.facebook.com/IEEEINSL/posts/here-we-present-to-you-the-most-talented-semi-finalists-whose-hard-work-dedicati/3027737500833258/</t>
-  </si>
-  <si>
-    <t>Winners: Pentathlon 2022</t>
-  </si>
-  <si>
-    <t>An inter-university article-writing competition hosted by MoraSpirit, a premier sports network.</t>
-  </si>
-  <si>
-    <t>thumbs/5.webp</t>
-  </si>
-  <si>
-    <t>https://www.facebook.com/MoraSpirit/posts/after-a-close-competition-between-all-the-participants-we-are-pleased-to-inform-/424187246412243/</t>
-  </si>
-  <si>
-    <t>Climate Crisis and Clean Energy</t>
-  </si>
-  <si>
-    <t>Article on the Severity of the Climate Crisis. Competition organized by the IEEE SLTC.</t>
-  </si>
-  <si>
-    <t>thumbs/4.webp</t>
-  </si>
-  <si>
-    <t>https://www.facebook.com/photo?fbid=1106724503145581&amp;set=a.1106720086479356</t>
-  </si>
-  <si>
-    <t>Clean Energy</t>
-  </si>
-  <si>
-    <t>Top 8: Most Popular Schoolboy Cricketers</t>
-  </si>
-  <si>
-    <t>batsman.lk nominee based on performers at the All-Island School's Cricket Tournament (D2) 2019</t>
-  </si>
-  <si>
-    <t>thumbs/3.webp</t>
-  </si>
-  <si>
-    <t>https://www.facebook.com/reel/2660611044253733</t>
-  </si>
-  <si>
-    <t>Stats Alert: 176 Runs vs Royal Panadura</t>
-  </si>
-  <si>
-    <t>"Vishal Perera's 176 was the highlight for the Wattala boys in that game."</t>
-  </si>
-  <si>
-    <t>thumbs/2.webp</t>
-  </si>
-  <si>
-    <t>https://www.thepapare.com/u19-schools-cricket-division-2-1st-week-of-january-2020-roundup/</t>
-  </si>
-  <si>
-    <t>Daily News: 176 Runs vs Royal Panadura</t>
-  </si>
-  <si>
-    <t>"Vishal Perera skipper and right hand opener of LISW scored 176 runs in 202 balls…"</t>
-  </si>
-  <si>
-    <t>thumbs/1.webp</t>
-  </si>
-  <si>
-    <t>Africa's premier virtual forum on space futures, innovation and collaboration.</t>
-  </si>
-  <si>
-    <t>Distinguished Panelist: SPACE UNGANA '26</t>
-  </si>
-  <si>
-    <t>SEDS KDU: SEDS SL's Best Local Chapter</t>
-  </si>
-  <si>
-    <t>Best Research Project: Aero Engineering</t>
+    <t>Project 8/8-1.webp</t>
+  </si>
+  <si>
+    <t>Project 8/8-1.webp|Project 8/8-2.webp|Project 8/8-3.webp|Project 8/8-4.webp</t>
+  </si>
+  <si>
+    <t>Coming soon…</t>
   </si>
 </sst>
 </file>
@@ -1370,8 +1382,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3137,7 +3150,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="2.6328125" bestFit="1" customWidth="1"/>
@@ -3176,178 +3189,201 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>219</v>
+        <v>418</v>
       </c>
       <c r="C2" t="s">
-        <v>220</v>
-      </c>
-      <c r="D2" t="s">
+        <v>428</v>
+      </c>
+      <c r="E2" t="s">
         <v>221</v>
       </c>
-      <c r="E2" t="s">
-        <v>222</v>
-      </c>
       <c r="F2" t="s">
-        <v>223</v>
+        <v>426</v>
       </c>
       <c r="G2" t="s">
-        <v>224</v>
+        <v>427</v>
       </c>
       <c r="H2" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C3" t="s">
-        <v>227</v>
-      </c>
-      <c r="D3" t="s">
-        <v>228</v>
+        <v>220</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>421</v>
       </c>
       <c r="E3" t="s">
+        <v>221</v>
+      </c>
+      <c r="F3" t="s">
         <v>222</v>
       </c>
-      <c r="F3" t="s">
-        <v>229</v>
-      </c>
       <c r="G3" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="H3" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
       <c r="C4" t="s">
-        <v>233</v>
-      </c>
-      <c r="D4" t="s">
-        <v>234</v>
+        <v>226</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>422</v>
       </c>
       <c r="E4" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="F4" t="s">
-        <v>235</v>
+        <v>227</v>
       </c>
       <c r="G4" t="s">
-        <v>236</v>
+        <v>228</v>
       </c>
       <c r="H4" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>237</v>
+        <v>419</v>
       </c>
       <c r="C5" t="s">
-        <v>238</v>
-      </c>
-      <c r="D5" t="s">
-        <v>239</v>
+        <v>230</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>423</v>
       </c>
       <c r="E5" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="F5" t="s">
-        <v>240</v>
+        <v>231</v>
       </c>
       <c r="G5" t="s">
-        <v>240</v>
+        <v>232</v>
       </c>
       <c r="H5" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>241</v>
+        <v>420</v>
       </c>
       <c r="C6" t="s">
-        <v>242</v>
+        <v>233</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>424</v>
       </c>
       <c r="E6" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="F6" t="s">
-        <v>243</v>
+        <v>234</v>
       </c>
       <c r="G6" t="s">
-        <v>244</v>
+        <v>234</v>
       </c>
       <c r="H6" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B7" t="s">
-        <v>245</v>
+        <v>235</v>
       </c>
       <c r="C7" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
       <c r="E7" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="F7" t="s">
-        <v>247</v>
+        <v>237</v>
       </c>
       <c r="G7" t="s">
-        <v>247</v>
+        <v>238</v>
       </c>
       <c r="H7" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8">
+        <v>2</v>
+      </c>
+      <c r="B8" t="s">
+        <v>239</v>
+      </c>
+      <c r="C8" t="s">
+        <v>240</v>
+      </c>
+      <c r="E8" t="s">
+        <v>221</v>
+      </c>
+      <c r="F8" t="s">
+        <v>241</v>
+      </c>
+      <c r="G8" t="s">
+        <v>241</v>
+      </c>
+      <c r="H8" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A9">
         <v>1</v>
       </c>
-      <c r="B8" t="s">
-        <v>248</v>
-      </c>
-      <c r="C8" t="s">
-        <v>249</v>
-      </c>
-      <c r="D8" t="s">
-        <v>250</v>
-      </c>
-      <c r="E8" t="s">
-        <v>251</v>
-      </c>
-      <c r="F8" t="s">
-        <v>252</v>
-      </c>
-      <c r="G8" t="s">
-        <v>253</v>
-      </c>
-      <c r="H8" t="s">
-        <v>231</v>
+      <c r="B9" t="s">
+        <v>242</v>
+      </c>
+      <c r="C9" t="s">
+        <v>243</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>425</v>
+      </c>
+      <c r="E9" t="s">
+        <v>244</v>
+      </c>
+      <c r="F9" t="s">
+        <v>245</v>
+      </c>
+      <c r="G9" t="s">
+        <v>246</v>
+      </c>
+      <c r="H9" t="s">
+        <v>229</v>
       </c>
     </row>
   </sheetData>
@@ -3378,22 +3414,22 @@
         <v>194</v>
       </c>
       <c r="C1" t="s">
-        <v>254</v>
+        <v>247</v>
       </c>
       <c r="D1" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="E1" t="s">
         <v>217</v>
       </c>
       <c r="F1" t="s">
-        <v>256</v>
+        <v>249</v>
       </c>
       <c r="G1" t="s">
-        <v>257</v>
+        <v>250</v>
       </c>
       <c r="H1" t="s">
-        <v>258</v>
+        <v>251</v>
       </c>
       <c r="I1" t="s">
         <v>22</v>
@@ -3404,10 +3440,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>259</v>
+        <v>252</v>
       </c>
       <c r="C2" t="s">
-        <v>260</v>
+        <v>253</v>
       </c>
       <c r="E2" t="str">
         <f t="shared" ref="E2:E33" si="0">"thumbs/" &amp; B2 &amp; ".webp"</f>
@@ -3418,13 +3454,13 @@
         <v>pdfs/Master of Arts - Space Entrepreneurship.pdf</v>
       </c>
       <c r="G2" t="s">
-        <v>261</v>
+        <v>254</v>
       </c>
       <c r="H2" t="s">
-        <v>260</v>
+        <v>253</v>
       </c>
       <c r="I2" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.35">
@@ -3432,10 +3468,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>262</v>
+        <v>255</v>
       </c>
       <c r="C3" t="s">
-        <v>260</v>
+        <v>253</v>
       </c>
       <c r="E3" t="str">
         <f t="shared" si="0"/>
@@ -3446,10 +3482,10 @@
         <v>pdfs/Acceptance Letter - EIIS.pdf</v>
       </c>
       <c r="G3" t="s">
-        <v>261</v>
+        <v>254</v>
       </c>
       <c r="H3" t="s">
-        <v>260</v>
+        <v>253</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.35">
@@ -3457,13 +3493,13 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>263</v>
+        <v>256</v>
       </c>
       <c r="C4" t="s">
-        <v>264</v>
+        <v>257</v>
       </c>
       <c r="D4" t="s">
-        <v>265</v>
+        <v>258</v>
       </c>
       <c r="E4" t="str">
         <f t="shared" si="0"/>
@@ -3474,13 +3510,13 @@
         <v>pdfs/Digitalisation in Aeronautics.pdf</v>
       </c>
       <c r="G4" t="s">
-        <v>266</v>
+        <v>259</v>
       </c>
       <c r="H4" t="s">
-        <v>267</v>
+        <v>260</v>
       </c>
       <c r="I4" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.35">
@@ -3488,13 +3524,13 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>268</v>
+        <v>261</v>
       </c>
       <c r="C5" t="s">
-        <v>264</v>
+        <v>257</v>
       </c>
       <c r="D5" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
       <c r="E5" t="str">
         <f t="shared" si="0"/>
@@ -3505,13 +3541,13 @@
         <v>pdfs/Digitalisation in Space Research.pdf</v>
       </c>
       <c r="G5" t="s">
-        <v>266</v>
+        <v>259</v>
       </c>
       <c r="H5" t="s">
-        <v>267</v>
+        <v>260</v>
       </c>
       <c r="I5" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.35">
@@ -3519,13 +3555,13 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>270</v>
+        <v>263</v>
       </c>
       <c r="C6" t="s">
+        <v>257</v>
+      </c>
+      <c r="D6" t="s">
         <v>264</v>
-      </c>
-      <c r="D6" t="s">
-        <v>271</v>
       </c>
       <c r="E6" t="str">
         <f t="shared" si="0"/>
@@ -3536,13 +3572,13 @@
         <v>pdfs/Digitalisation in the Aerospace Industry.pdf</v>
       </c>
       <c r="G6" t="s">
-        <v>266</v>
+        <v>259</v>
       </c>
       <c r="H6" t="s">
-        <v>267</v>
+        <v>260</v>
       </c>
       <c r="I6" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.35">
@@ -3550,13 +3586,13 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>272</v>
+        <v>265</v>
       </c>
       <c r="C7" t="s">
-        <v>273</v>
+        <v>266</v>
       </c>
       <c r="D7" t="s">
-        <v>274</v>
+        <v>267</v>
       </c>
       <c r="E7" t="str">
         <f t="shared" si="0"/>
@@ -3567,10 +3603,10 @@
         <v>pdfs/Aerospace Materials.pdf</v>
       </c>
       <c r="G7" t="s">
-        <v>266</v>
+        <v>259</v>
       </c>
       <c r="I7" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.35">
@@ -3578,13 +3614,13 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>275</v>
+        <v>268</v>
       </c>
       <c r="C8" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
       <c r="D8" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
       <c r="E8" t="str">
         <f t="shared" si="0"/>
@@ -3595,10 +3631,10 @@
         <v>pdfs/Robotics - Aerial Robotics.pdf</v>
       </c>
       <c r="G8" t="s">
-        <v>266</v>
+        <v>259</v>
       </c>
       <c r="I8" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.35">
@@ -3606,10 +3642,10 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>278</v>
+        <v>271</v>
       </c>
       <c r="C9" t="s">
-        <v>279</v>
+        <v>272</v>
       </c>
       <c r="E9" t="str">
         <f t="shared" si="0"/>
@@ -3620,7 +3656,7 @@
         <v>pdfs/Best Research Project.pdf</v>
       </c>
       <c r="I9" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.35">
@@ -3628,10 +3664,10 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>280</v>
+        <v>273</v>
       </c>
       <c r="C10" t="s">
-        <v>281</v>
+        <v>274</v>
       </c>
       <c r="E10" t="str">
         <f t="shared" si="0"/>
@@ -3642,10 +3678,10 @@
         <v>pdfs/Best Poster Presentation.pdf</v>
       </c>
       <c r="G10" t="s">
-        <v>266</v>
+        <v>259</v>
       </c>
       <c r="I10" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.35">
@@ -3653,10 +3689,10 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>282</v>
+        <v>275</v>
       </c>
       <c r="C11" t="s">
-        <v>281</v>
+        <v>274</v>
       </c>
       <c r="E11" t="str">
         <f t="shared" si="0"/>
@@ -3667,10 +3703,10 @@
         <v>pdfs/Paper Presentation at IRC.pdf</v>
       </c>
       <c r="G11" t="s">
-        <v>266</v>
+        <v>259</v>
       </c>
       <c r="I11" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.35">
@@ -3678,10 +3714,10 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>283</v>
+        <v>276</v>
       </c>
       <c r="C12" t="s">
-        <v>279</v>
+        <v>272</v>
       </c>
       <c r="E12" t="str">
         <f t="shared" si="0"/>
@@ -3692,13 +3728,13 @@
         <v>pdfs/BSc. (Hons) Aeronautical Engineering.pdf</v>
       </c>
       <c r="G12" t="s">
-        <v>266</v>
+        <v>259</v>
       </c>
       <c r="H12" t="s">
-        <v>284</v>
+        <v>277</v>
       </c>
       <c r="I12" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.35">
@@ -3706,7 +3742,7 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>285</v>
+        <v>278</v>
       </c>
       <c r="C13" t="s">
         <v>161</v>
@@ -3720,13 +3756,13 @@
         <v>pdfs/Chairperson - SEDS SL.pdf</v>
       </c>
       <c r="G13" t="s">
-        <v>266</v>
+        <v>259</v>
       </c>
       <c r="H13" t="s">
-        <v>284</v>
+        <v>277</v>
       </c>
       <c r="I13" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.35">
@@ -3734,10 +3770,10 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>286</v>
+        <v>279</v>
       </c>
       <c r="C14" t="s">
-        <v>279</v>
+        <v>272</v>
       </c>
       <c r="E14" t="str">
         <f t="shared" si="0"/>
@@ -3748,10 +3784,10 @@
         <v>pdfs/President - SEDS KDU.pdf</v>
       </c>
       <c r="G14" t="s">
-        <v>266</v>
+        <v>259</v>
       </c>
       <c r="I14" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.35">
@@ -3759,7 +3795,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>287</v>
+        <v>280</v>
       </c>
       <c r="C15" t="s">
         <v>166</v>
@@ -3773,10 +3809,10 @@
         <v>pdfs/Service Letter.pdf</v>
       </c>
       <c r="G15" t="s">
-        <v>266</v>
+        <v>259</v>
       </c>
       <c r="I15" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.35">
@@ -3784,13 +3820,13 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>288</v>
+        <v>281</v>
       </c>
       <c r="C16" t="s">
-        <v>289</v>
+        <v>282</v>
       </c>
       <c r="D16" t="s">
-        <v>290</v>
+        <v>283</v>
       </c>
       <c r="E16" t="str">
         <f t="shared" si="0"/>
@@ -3801,10 +3837,10 @@
         <v>pdfs/Semi-Finalists - IEEE INSL 2021.pdf</v>
       </c>
       <c r="G16" t="s">
-        <v>291</v>
+        <v>284</v>
       </c>
       <c r="I16" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.35">
@@ -3812,10 +3848,10 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>292</v>
+        <v>285</v>
       </c>
       <c r="C17" t="s">
-        <v>279</v>
+        <v>272</v>
       </c>
       <c r="E17" t="str">
         <f t="shared" si="0"/>
@@ -3826,10 +3862,10 @@
         <v>pdfs/Inter-Faculty Cricket (2022).pdf</v>
       </c>
       <c r="G17" t="s">
-        <v>293</v>
+        <v>286</v>
       </c>
       <c r="I17" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.35">
@@ -3837,10 +3873,10 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>294</v>
+        <v>287</v>
       </c>
       <c r="C18" t="s">
-        <v>279</v>
+        <v>272</v>
       </c>
       <c r="E18" t="str">
         <f t="shared" si="0"/>
@@ -3851,10 +3887,10 @@
         <v>pdfs/Inter-Faculty Cricket (2023).pdf</v>
       </c>
       <c r="G18" t="s">
-        <v>293</v>
+        <v>286</v>
       </c>
       <c r="I18" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.35">
@@ -3862,10 +3898,10 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>295</v>
+        <v>288</v>
       </c>
       <c r="C19" t="s">
-        <v>279</v>
+        <v>272</v>
       </c>
       <c r="E19" t="str">
         <f t="shared" si="0"/>
@@ -3876,10 +3912,10 @@
         <v>pdfs/Leadership Program (2020).pdf</v>
       </c>
       <c r="G19" t="s">
-        <v>296</v>
+        <v>289</v>
       </c>
       <c r="I19" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.35">
@@ -3887,10 +3923,10 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>297</v>
+        <v>290</v>
       </c>
       <c r="C20" t="s">
-        <v>279</v>
+        <v>272</v>
       </c>
       <c r="E20" t="str">
         <f t="shared" si="0"/>
@@ -3901,10 +3937,10 @@
         <v>pdfs/Leadership Program (2017).pdf</v>
       </c>
       <c r="G20" t="s">
-        <v>296</v>
+        <v>289</v>
       </c>
       <c r="I20" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.35">
@@ -3912,13 +3948,13 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>298</v>
+        <v>291</v>
       </c>
       <c r="C21" t="s">
-        <v>299</v>
+        <v>292</v>
       </c>
       <c r="D21" t="s">
-        <v>300</v>
+        <v>293</v>
       </c>
       <c r="E21" t="str">
         <f t="shared" si="0"/>
@@ -3929,13 +3965,13 @@
         <v>pdfs/Foundations of Project Management.pdf</v>
       </c>
       <c r="G21" t="s">
-        <v>296</v>
+        <v>289</v>
       </c>
       <c r="H21" t="s">
-        <v>301</v>
+        <v>294</v>
       </c>
       <c r="I21" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.35">
@@ -3943,13 +3979,13 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>302</v>
+        <v>295</v>
       </c>
       <c r="C22" t="s">
-        <v>299</v>
+        <v>292</v>
       </c>
       <c r="D22" t="s">
-        <v>303</v>
+        <v>296</v>
       </c>
       <c r="E22" t="str">
         <f t="shared" si="0"/>
@@ -3960,13 +3996,13 @@
         <v>pdfs/Project Initiation - Starting a Successful Project.pdf</v>
       </c>
       <c r="G22" t="s">
-        <v>296</v>
+        <v>289</v>
       </c>
       <c r="H22" t="s">
-        <v>301</v>
+        <v>294</v>
       </c>
       <c r="I22" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.35">
@@ -3974,13 +4010,13 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>304</v>
+        <v>297</v>
       </c>
       <c r="C23" t="s">
-        <v>299</v>
+        <v>292</v>
       </c>
       <c r="D23" t="s">
-        <v>305</v>
+        <v>298</v>
       </c>
       <c r="E23" t="str">
         <f t="shared" si="0"/>
@@ -3991,13 +4027,13 @@
         <v>pdfs/Project Planning - Putting It All Together.pdf</v>
       </c>
       <c r="G23" t="s">
-        <v>296</v>
+        <v>289</v>
       </c>
       <c r="H23" t="s">
-        <v>301</v>
+        <v>294</v>
       </c>
       <c r="I23" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.35">
@@ -4005,13 +4041,13 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>306</v>
+        <v>299</v>
       </c>
       <c r="C24" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
       <c r="D24" t="s">
-        <v>307</v>
+        <v>300</v>
       </c>
       <c r="E24" t="str">
         <f t="shared" si="0"/>
@@ -4022,10 +4058,10 @@
         <v>pdfs/Introduction to Marketing.pdf</v>
       </c>
       <c r="G24" t="s">
-        <v>291</v>
+        <v>284</v>
       </c>
       <c r="I24" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.35">
@@ -4033,10 +4069,10 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>308</v>
+        <v>301</v>
       </c>
       <c r="C25" t="s">
-        <v>299</v>
+        <v>292</v>
       </c>
       <c r="E25" t="str">
         <f t="shared" si="0"/>
@@ -4047,10 +4083,10 @@
         <v>pdfs/Fundamentals of Digital Marketing.pdf</v>
       </c>
       <c r="G25" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="I25" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.35">
@@ -4058,13 +4094,13 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>310</v>
+        <v>303</v>
       </c>
       <c r="C26" t="s">
-        <v>311</v>
+        <v>304</v>
       </c>
       <c r="D26" t="s">
-        <v>312</v>
+        <v>305</v>
       </c>
       <c r="E26" t="str">
         <f t="shared" si="0"/>
@@ -4075,13 +4111,13 @@
         <v>pdfs/Claude 101.pdf</v>
       </c>
       <c r="G26" t="s">
-        <v>313</v>
+        <v>306</v>
       </c>
       <c r="H26" t="s">
-        <v>314</v>
+        <v>307</v>
       </c>
       <c r="I26" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.35">
@@ -4089,13 +4125,13 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>315</v>
+        <v>308</v>
       </c>
       <c r="C27" t="s">
-        <v>311</v>
+        <v>304</v>
       </c>
       <c r="D27" t="s">
-        <v>316</v>
+        <v>309</v>
       </c>
       <c r="E27" t="str">
         <f t="shared" si="0"/>
@@ -4106,13 +4142,13 @@
         <v>pdfs/Claude Code 101.pdf</v>
       </c>
       <c r="G27" t="s">
-        <v>313</v>
+        <v>306</v>
       </c>
       <c r="H27" t="s">
-        <v>314</v>
+        <v>307</v>
       </c>
       <c r="I27" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.35">
@@ -4120,13 +4156,13 @@
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>317</v>
+        <v>310</v>
       </c>
       <c r="C28" t="s">
+        <v>304</v>
+      </c>
+      <c r="D28" t="s">
         <v>311</v>
-      </c>
-      <c r="D28" t="s">
-        <v>318</v>
       </c>
       <c r="E28" t="str">
         <f t="shared" si="0"/>
@@ -4137,13 +4173,13 @@
         <v>pdfs/Claude Platform 101.pdf</v>
       </c>
       <c r="G28" t="s">
-        <v>313</v>
+        <v>306</v>
       </c>
       <c r="H28" t="s">
-        <v>314</v>
+        <v>307</v>
       </c>
       <c r="I28" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.35">
@@ -4151,13 +4187,13 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>319</v>
+        <v>312</v>
       </c>
       <c r="C29" t="s">
-        <v>311</v>
+        <v>304</v>
       </c>
       <c r="D29" t="s">
-        <v>320</v>
+        <v>313</v>
       </c>
       <c r="E29" t="str">
         <f t="shared" si="0"/>
@@ -4168,13 +4204,13 @@
         <v>pdfs/Introduction to Claude Cowork.pdf</v>
       </c>
       <c r="G29" t="s">
-        <v>313</v>
+        <v>306</v>
       </c>
       <c r="H29" t="s">
-        <v>314</v>
+        <v>307</v>
       </c>
       <c r="I29" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.35">
@@ -4182,13 +4218,13 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
       <c r="C30" t="s">
-        <v>311</v>
+        <v>304</v>
       </c>
       <c r="D30" t="s">
-        <v>322</v>
+        <v>315</v>
       </c>
       <c r="E30" t="str">
         <f t="shared" si="0"/>
@@ -4199,13 +4235,13 @@
         <v>pdfs/Claude Code in Action.pdf</v>
       </c>
       <c r="G30" t="s">
-        <v>313</v>
+        <v>306</v>
       </c>
       <c r="H30" t="s">
-        <v>314</v>
+        <v>307</v>
       </c>
       <c r="I30" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.35">
@@ -4213,13 +4249,13 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>323</v>
+        <v>316</v>
       </c>
       <c r="C31" t="s">
-        <v>311</v>
+        <v>304</v>
       </c>
       <c r="D31" t="s">
-        <v>324</v>
+        <v>317</v>
       </c>
       <c r="E31" t="str">
         <f t="shared" si="0"/>
@@ -4230,13 +4266,13 @@
         <v>pdfs/AI Fluency - Frameworks &amp; Foundations.pdf</v>
       </c>
       <c r="G31" t="s">
-        <v>313</v>
+        <v>306</v>
       </c>
       <c r="H31" t="s">
-        <v>314</v>
+        <v>307</v>
       </c>
       <c r="I31" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.35">
@@ -4244,13 +4280,13 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>325</v>
+        <v>318</v>
       </c>
       <c r="C32" t="s">
-        <v>311</v>
+        <v>304</v>
       </c>
       <c r="D32" t="s">
-        <v>326</v>
+        <v>319</v>
       </c>
       <c r="E32" t="str">
         <f t="shared" si="0"/>
@@ -4261,13 +4297,13 @@
         <v>pdfs/Introduction to Model Context Protocol.pdf</v>
       </c>
       <c r="G32" t="s">
-        <v>313</v>
+        <v>306</v>
       </c>
       <c r="H32" t="s">
-        <v>314</v>
+        <v>307</v>
       </c>
       <c r="I32" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.35">
@@ -4275,13 +4311,13 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>327</v>
+        <v>320</v>
       </c>
       <c r="C33" t="s">
-        <v>311</v>
+        <v>304</v>
       </c>
       <c r="D33" t="s">
-        <v>328</v>
+        <v>321</v>
       </c>
       <c r="E33" t="str">
         <f t="shared" si="0"/>
@@ -4292,13 +4328,13 @@
         <v>pdfs/Model Context Protocol - Advanced Topics.pdf</v>
       </c>
       <c r="G33" t="s">
-        <v>313</v>
+        <v>306</v>
       </c>
       <c r="H33" t="s">
-        <v>314</v>
+        <v>307</v>
       </c>
       <c r="I33" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.35">
@@ -4306,13 +4342,13 @@
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>329</v>
+        <v>322</v>
       </c>
       <c r="C34" t="s">
-        <v>311</v>
+        <v>304</v>
       </c>
       <c r="D34" t="s">
-        <v>330</v>
+        <v>323</v>
       </c>
       <c r="E34" t="str">
         <f t="shared" ref="E34:E52" si="2">"thumbs/" &amp; B34 &amp; ".webp"</f>
@@ -4323,13 +4359,13 @@
         <v>pdfs/AI Fluency for Educators.pdf</v>
       </c>
       <c r="G34" t="s">
-        <v>313</v>
+        <v>306</v>
       </c>
       <c r="H34" t="s">
-        <v>314</v>
+        <v>307</v>
       </c>
       <c r="I34" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.35">
@@ -4337,13 +4373,13 @@
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>331</v>
+        <v>324</v>
       </c>
       <c r="C35" t="s">
-        <v>311</v>
+        <v>304</v>
       </c>
       <c r="D35" t="s">
-        <v>332</v>
+        <v>325</v>
       </c>
       <c r="E35" t="str">
         <f t="shared" si="2"/>
@@ -4354,13 +4390,13 @@
         <v>pdfs/AI Fluency for Students.pdf</v>
       </c>
       <c r="G35" t="s">
-        <v>313</v>
+        <v>306</v>
       </c>
       <c r="H35" t="s">
-        <v>314</v>
+        <v>307</v>
       </c>
       <c r="I35" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.35">
@@ -4368,13 +4404,13 @@
         <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>333</v>
+        <v>326</v>
       </c>
       <c r="C36" t="s">
-        <v>311</v>
+        <v>304</v>
       </c>
       <c r="D36" t="s">
-        <v>334</v>
+        <v>327</v>
       </c>
       <c r="E36" t="str">
         <f t="shared" si="2"/>
@@ -4385,13 +4421,13 @@
         <v>pdfs/Teaching the AI Fluency Framework.pdf</v>
       </c>
       <c r="G36" t="s">
-        <v>313</v>
+        <v>306</v>
       </c>
       <c r="H36" t="s">
-        <v>314</v>
+        <v>307</v>
       </c>
       <c r="I36" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.35">
@@ -4399,13 +4435,13 @@
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>335</v>
+        <v>328</v>
       </c>
       <c r="C37" t="s">
-        <v>311</v>
+        <v>304</v>
       </c>
       <c r="D37" t="s">
-        <v>336</v>
+        <v>329</v>
       </c>
       <c r="E37" t="str">
         <f t="shared" si="2"/>
@@ -4416,13 +4452,13 @@
         <v>pdfs/AI Fluency for Non-Profits.pdf</v>
       </c>
       <c r="G37" t="s">
-        <v>313</v>
+        <v>306</v>
       </c>
       <c r="H37" t="s">
-        <v>314</v>
+        <v>307</v>
       </c>
       <c r="I37" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.35">
@@ -4430,13 +4466,13 @@
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>337</v>
+        <v>330</v>
       </c>
       <c r="C38" t="s">
-        <v>311</v>
+        <v>304</v>
       </c>
       <c r="D38" t="s">
-        <v>338</v>
+        <v>331</v>
       </c>
       <c r="E38" t="str">
         <f t="shared" si="2"/>
@@ -4447,13 +4483,13 @@
         <v>pdfs/AI Fluency for Small Businesses.pdf</v>
       </c>
       <c r="G38" t="s">
-        <v>313</v>
+        <v>306</v>
       </c>
       <c r="H38" t="s">
-        <v>314</v>
+        <v>307</v>
       </c>
       <c r="I38" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.35">
@@ -4461,13 +4497,13 @@
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>339</v>
+        <v>332</v>
       </c>
       <c r="C39" t="s">
-        <v>311</v>
+        <v>304</v>
       </c>
       <c r="D39" t="s">
-        <v>340</v>
+        <v>333</v>
       </c>
       <c r="E39" t="str">
         <f t="shared" si="2"/>
@@ -4478,13 +4514,13 @@
         <v>pdfs/Introduction to Agent Skills.pdf</v>
       </c>
       <c r="G39" t="s">
-        <v>313</v>
+        <v>306</v>
       </c>
       <c r="H39" t="s">
-        <v>314</v>
+        <v>307</v>
       </c>
       <c r="I39" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.35">
@@ -4492,13 +4528,13 @@
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>341</v>
+        <v>334</v>
       </c>
       <c r="C40" t="s">
-        <v>311</v>
+        <v>304</v>
       </c>
       <c r="D40" t="s">
-        <v>342</v>
+        <v>335</v>
       </c>
       <c r="E40" t="str">
         <f t="shared" si="2"/>
@@ -4509,13 +4545,13 @@
         <v>pdfs/Introduction to Sub-Agents.pdf</v>
       </c>
       <c r="G40" t="s">
-        <v>313</v>
+        <v>306</v>
       </c>
       <c r="H40" t="s">
-        <v>314</v>
+        <v>307</v>
       </c>
       <c r="I40" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.35">
@@ -4523,13 +4559,13 @@
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>343</v>
+        <v>336</v>
       </c>
       <c r="C41" t="s">
-        <v>311</v>
+        <v>304</v>
       </c>
       <c r="D41" t="s">
-        <v>344</v>
+        <v>337</v>
       </c>
       <c r="E41" t="str">
         <f t="shared" si="2"/>
@@ -4540,13 +4576,13 @@
         <v>pdfs/AI Capabilities &amp; Limitations.pdf</v>
       </c>
       <c r="G41" t="s">
-        <v>313</v>
+        <v>306</v>
       </c>
       <c r="H41" t="s">
-        <v>314</v>
+        <v>307</v>
       </c>
       <c r="I41" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.35">
@@ -4554,13 +4590,13 @@
         <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>345</v>
+        <v>338</v>
       </c>
       <c r="C42" t="s">
-        <v>311</v>
+        <v>304</v>
       </c>
       <c r="D42" t="s">
-        <v>346</v>
+        <v>339</v>
       </c>
       <c r="E42" t="str">
         <f t="shared" si="2"/>
@@ -4571,13 +4607,13 @@
         <v>pdfs/Claude with Anthropic API.pdf</v>
       </c>
       <c r="G42" t="s">
-        <v>313</v>
+        <v>306</v>
       </c>
       <c r="H42" t="s">
-        <v>314</v>
+        <v>307</v>
       </c>
       <c r="I42" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.35">
@@ -4585,13 +4621,13 @@
         <v>42</v>
       </c>
       <c r="B43" t="s">
-        <v>347</v>
+        <v>340</v>
       </c>
       <c r="C43" t="s">
-        <v>311</v>
+        <v>304</v>
       </c>
       <c r="D43" t="s">
-        <v>348</v>
+        <v>341</v>
       </c>
       <c r="E43" t="str">
         <f t="shared" si="2"/>
@@ -4602,13 +4638,13 @@
         <v>pdfs/Claude with Google Vertex AI.pdf</v>
       </c>
       <c r="G43" t="s">
-        <v>313</v>
+        <v>306</v>
       </c>
       <c r="H43" t="s">
-        <v>314</v>
+        <v>307</v>
       </c>
       <c r="I43" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.35">
@@ -4616,13 +4652,13 @@
         <v>43</v>
       </c>
       <c r="B44" t="s">
-        <v>349</v>
+        <v>342</v>
       </c>
       <c r="C44" t="s">
-        <v>311</v>
+        <v>304</v>
       </c>
       <c r="D44" t="s">
-        <v>350</v>
+        <v>343</v>
       </c>
       <c r="E44" t="str">
         <f t="shared" si="2"/>
@@ -4633,13 +4669,13 @@
         <v>pdfs/Claude with Amazon Bedrock.pdf</v>
       </c>
       <c r="G44" t="s">
-        <v>313</v>
+        <v>306</v>
       </c>
       <c r="H44" t="s">
-        <v>314</v>
+        <v>307</v>
       </c>
       <c r="I44" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.35">
@@ -4647,13 +4683,13 @@
         <v>44</v>
       </c>
       <c r="B45" t="s">
-        <v>351</v>
+        <v>344</v>
       </c>
       <c r="C45" t="s">
-        <v>352</v>
+        <v>345</v>
       </c>
       <c r="D45" t="s">
-        <v>353</v>
+        <v>346</v>
       </c>
       <c r="E45" t="str">
         <f t="shared" si="2"/>
@@ -4664,10 +4700,10 @@
         <v>pdfs/Getting Started with Python.pdf</v>
       </c>
       <c r="G45" t="s">
-        <v>354</v>
+        <v>347</v>
       </c>
       <c r="I45" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.35">
@@ -4675,10 +4711,10 @@
         <v>45</v>
       </c>
       <c r="B46" t="s">
-        <v>355</v>
+        <v>348</v>
       </c>
       <c r="C46" t="s">
-        <v>356</v>
+        <v>349</v>
       </c>
       <c r="E46" t="str">
         <f t="shared" si="2"/>
@@ -4689,10 +4725,10 @@
         <v>pdfs/Gampaha District Cricket Team.pdf</v>
       </c>
       <c r="G46" t="s">
-        <v>293</v>
+        <v>286</v>
       </c>
       <c r="I46" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.35">
@@ -4700,7 +4736,7 @@
         <v>46</v>
       </c>
       <c r="B47" t="s">
-        <v>357</v>
+        <v>350</v>
       </c>
       <c r="C47" t="s">
         <v>196</v>
@@ -4714,10 +4750,10 @@
         <v>pdfs/Sports Colors - Cricket.pdf</v>
       </c>
       <c r="G47" t="s">
-        <v>293</v>
+        <v>286</v>
       </c>
       <c r="I47" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.35">
@@ -4725,10 +4761,10 @@
         <v>47</v>
       </c>
       <c r="B48" t="s">
-        <v>358</v>
+        <v>351</v>
       </c>
       <c r="C48" t="s">
-        <v>359</v>
+        <v>352</v>
       </c>
       <c r="E48" t="str">
         <f t="shared" si="2"/>
@@ -4739,10 +4775,10 @@
         <v>pdfs/All-Island U19 DIII Semi-Finalists (2019).pdf</v>
       </c>
       <c r="G48" t="s">
-        <v>293</v>
+        <v>286</v>
       </c>
       <c r="I48" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.35">
@@ -4750,7 +4786,7 @@
         <v>48</v>
       </c>
       <c r="B49" t="s">
-        <v>360</v>
+        <v>353</v>
       </c>
       <c r="C49" t="s">
         <v>196</v>
@@ -4764,10 +4800,10 @@
         <v>pdfs/School Leaving Certificate.pdf</v>
       </c>
       <c r="G49" t="s">
-        <v>361</v>
+        <v>354</v>
       </c>
       <c r="I49" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.35">
@@ -4775,7 +4811,7 @@
         <v>49</v>
       </c>
       <c r="B50" t="s">
-        <v>362</v>
+        <v>355</v>
       </c>
       <c r="C50" t="s">
         <v>196</v>
@@ -4789,10 +4825,10 @@
         <v>pdfs/Character Certificate.pdf</v>
       </c>
       <c r="G50" t="s">
-        <v>361</v>
+        <v>354</v>
       </c>
       <c r="I50" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.35">
@@ -4800,10 +4836,10 @@
         <v>50</v>
       </c>
       <c r="B51" t="s">
-        <v>363</v>
+        <v>356</v>
       </c>
       <c r="C51" t="s">
-        <v>364</v>
+        <v>357</v>
       </c>
       <c r="E51" t="str">
         <f t="shared" si="2"/>
@@ -4814,10 +4850,10 @@
         <v>pdfs/Advanced Level Results.pdf</v>
       </c>
       <c r="G51" t="s">
-        <v>361</v>
+        <v>354</v>
       </c>
       <c r="I51" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.35">
@@ -4825,10 +4861,10 @@
         <v>51</v>
       </c>
       <c r="B52" t="s">
-        <v>365</v>
+        <v>358</v>
       </c>
       <c r="C52" t="s">
-        <v>366</v>
+        <v>359</v>
       </c>
       <c r="E52" t="str">
         <f t="shared" si="2"/>
@@ -4839,10 +4875,10 @@
         <v>pdfs/IGCSE OL Results.pdf</v>
       </c>
       <c r="G52" t="s">
-        <v>361</v>
+        <v>354</v>
       </c>
       <c r="I52" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
   </sheetData>
@@ -4872,7 +4908,7 @@
         <v>217</v>
       </c>
       <c r="E1" t="s">
-        <v>367</v>
+        <v>360</v>
       </c>
       <c r="F1" t="s">
         <v>216</v>
@@ -4886,22 +4922,22 @@
         <v>14</v>
       </c>
       <c r="B2" t="s">
-        <v>422</v>
+        <v>415</v>
       </c>
       <c r="C2" t="s">
-        <v>421</v>
+        <v>414</v>
       </c>
       <c r="D2" t="s">
-        <v>368</v>
+        <v>361</v>
       </c>
       <c r="E2" t="s">
-        <v>369</v>
+        <v>362</v>
       </c>
       <c r="F2" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="G2" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
@@ -4909,22 +4945,22 @@
         <v>13</v>
       </c>
       <c r="B3" t="s">
-        <v>370</v>
+        <v>363</v>
       </c>
       <c r="C3" t="s">
-        <v>371</v>
+        <v>364</v>
       </c>
       <c r="D3" t="s">
-        <v>372</v>
+        <v>365</v>
       </c>
       <c r="E3" t="s">
-        <v>373</v>
+        <v>366</v>
       </c>
       <c r="F3" t="s">
-        <v>374</v>
+        <v>367</v>
       </c>
       <c r="G3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
@@ -4932,22 +4968,22 @@
         <v>12</v>
       </c>
       <c r="B4" t="s">
-        <v>423</v>
+        <v>416</v>
       </c>
       <c r="C4" t="s">
-        <v>375</v>
+        <v>368</v>
       </c>
       <c r="D4" t="s">
-        <v>376</v>
+        <v>369</v>
       </c>
       <c r="E4" t="s">
-        <v>377</v>
+        <v>370</v>
       </c>
       <c r="F4" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="G4" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
@@ -4955,22 +4991,22 @@
         <v>11</v>
       </c>
       <c r="B5" t="s">
-        <v>378</v>
+        <v>371</v>
       </c>
       <c r="C5" t="s">
-        <v>379</v>
+        <v>372</v>
       </c>
       <c r="D5" t="s">
-        <v>380</v>
+        <v>373</v>
       </c>
       <c r="E5" t="s">
-        <v>381</v>
+        <v>374</v>
       </c>
       <c r="F5" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="G5" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
@@ -4978,22 +5014,22 @@
         <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>424</v>
+        <v>417</v>
       </c>
       <c r="C6" t="s">
-        <v>382</v>
+        <v>375</v>
       </c>
       <c r="D6" t="s">
-        <v>383</v>
+        <v>376</v>
       </c>
       <c r="E6" t="s">
-        <v>384</v>
+        <v>377</v>
       </c>
       <c r="F6" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="G6" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
@@ -5001,22 +5037,22 @@
         <v>9</v>
       </c>
       <c r="B7" t="s">
-        <v>385</v>
+        <v>378</v>
       </c>
       <c r="C7" t="s">
-        <v>386</v>
+        <v>379</v>
       </c>
       <c r="D7" t="s">
-        <v>387</v>
+        <v>380</v>
       </c>
       <c r="E7" t="s">
-        <v>388</v>
+        <v>381</v>
       </c>
       <c r="F7" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="G7" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
@@ -5024,22 +5060,22 @@
         <v>8</v>
       </c>
       <c r="B8" t="s">
-        <v>389</v>
+        <v>382</v>
       </c>
       <c r="C8" t="s">
-        <v>390</v>
+        <v>383</v>
       </c>
       <c r="D8" t="s">
-        <v>391</v>
+        <v>384</v>
       </c>
       <c r="E8" t="s">
-        <v>392</v>
+        <v>385</v>
       </c>
       <c r="F8" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="G8" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
@@ -5047,22 +5083,22 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>393</v>
+        <v>386</v>
       </c>
       <c r="C9" t="s">
-        <v>394</v>
+        <v>387</v>
       </c>
       <c r="D9" t="s">
-        <v>395</v>
+        <v>388</v>
       </c>
       <c r="E9" t="s">
-        <v>396</v>
+        <v>389</v>
       </c>
       <c r="F9" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="G9" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.35">
@@ -5070,22 +5106,22 @@
         <v>6</v>
       </c>
       <c r="B10" t="s">
-        <v>397</v>
+        <v>390</v>
       </c>
       <c r="C10" t="s">
-        <v>398</v>
+        <v>391</v>
       </c>
       <c r="D10" t="s">
-        <v>399</v>
+        <v>392</v>
       </c>
       <c r="E10" t="s">
-        <v>400</v>
+        <v>393</v>
       </c>
       <c r="F10" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
       <c r="G10" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
@@ -5093,22 +5129,22 @@
         <v>5</v>
       </c>
       <c r="B11" t="s">
-        <v>401</v>
+        <v>394</v>
       </c>
       <c r="C11" t="s">
-        <v>402</v>
+        <v>395</v>
       </c>
       <c r="D11" t="s">
-        <v>403</v>
+        <v>396</v>
       </c>
       <c r="E11" t="s">
-        <v>404</v>
+        <v>397</v>
       </c>
       <c r="F11" t="s">
-        <v>293</v>
+        <v>286</v>
       </c>
       <c r="G11" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.35">
@@ -5116,22 +5152,22 @@
         <v>4</v>
       </c>
       <c r="B12" t="s">
-        <v>405</v>
+        <v>398</v>
       </c>
       <c r="C12" t="s">
-        <v>406</v>
+        <v>399</v>
       </c>
       <c r="D12" t="s">
-        <v>407</v>
+        <v>400</v>
       </c>
       <c r="E12" t="s">
-        <v>408</v>
+        <v>401</v>
       </c>
       <c r="F12" t="s">
-        <v>409</v>
+        <v>402</v>
       </c>
       <c r="G12" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.35">
@@ -5139,22 +5175,22 @@
         <v>3</v>
       </c>
       <c r="B13" t="s">
-        <v>410</v>
+        <v>403</v>
       </c>
       <c r="C13" t="s">
-        <v>411</v>
+        <v>404</v>
       </c>
       <c r="D13" t="s">
-        <v>412</v>
+        <v>405</v>
       </c>
       <c r="E13" t="s">
-        <v>413</v>
+        <v>406</v>
       </c>
       <c r="F13" t="s">
-        <v>293</v>
+        <v>286</v>
       </c>
       <c r="G13" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.35">
@@ -5162,22 +5198,22 @@
         <v>2</v>
       </c>
       <c r="B14" t="s">
-        <v>414</v>
+        <v>407</v>
       </c>
       <c r="C14" t="s">
-        <v>415</v>
+        <v>408</v>
       </c>
       <c r="D14" t="s">
-        <v>416</v>
+        <v>409</v>
       </c>
       <c r="E14" t="s">
-        <v>417</v>
+        <v>410</v>
       </c>
       <c r="F14" t="s">
-        <v>293</v>
+        <v>286</v>
       </c>
       <c r="G14" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.35">
@@ -5185,22 +5221,22 @@
         <v>1</v>
       </c>
       <c r="B15" t="s">
-        <v>418</v>
+        <v>411</v>
       </c>
       <c r="C15" t="s">
-        <v>419</v>
+        <v>412</v>
       </c>
       <c r="D15" t="s">
-        <v>420</v>
+        <v>413</v>
       </c>
       <c r="E15" t="s">
-        <v>369</v>
+        <v>362</v>
       </c>
       <c r="F15" t="s">
-        <v>293</v>
+        <v>286</v>
       </c>
       <c r="G15" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Remove // MISSION BRIEF label from project cards
</commit_message>
<xml_diff>
--- a/fetch.xlsx
+++ b/fetch.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ghz\Documents\Claude\Projects\000 Online Portfolio - vcperera\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAAF3796-65EB-465C-8918-E8DA6A67B567}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF7755A7-8E62-44C7-8391-34FAB0B74207}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="757" uniqueCount="429">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="758" uniqueCount="430">
   <si>
     <t>ID</t>
   </si>
@@ -704,9 +704,6 @@
     <t>Aquila: An Energy Grid for Space</t>
   </si>
   <si>
-    <t>Winner: EIIS x Airbus Annual Space Entrepreneurship Challenge Solving the Space Debris Challenge in an Sustainable Manner</t>
-  </si>
-  <si>
     <t>Aerospace</t>
   </si>
   <si>
@@ -722,9 +719,6 @@
     <t>Aerodynamics of a Nano-Coated Flat Plate</t>
   </si>
   <si>
-    <t>Numeric Approach (CFD) | Winner: Best Poster Presentation, 16th International Research Conference (IRC)</t>
-  </si>
-  <si>
     <t>Project 6/6-1.webp</t>
   </si>
   <si>
@@ -734,18 +728,12 @@
     <t>YES</t>
   </si>
   <si>
-    <t>Numeric Approach (CFD) | Winner: Best Research Project (2024), Department of Aeronautical Engineering</t>
-  </si>
-  <si>
     <t>Project 5/5-1.webp</t>
   </si>
   <si>
     <t>Project 5/5-1.webp|Project 5/5-2.webp|Project 5/5-3.webp|Project 5/5-4.webp|Project 5/5-5.webp</t>
   </si>
   <si>
-    <t>Experimental Approach (Lab) | Grant of LKR 1Mn Approved by Combinatorial Advanced Research &amp; Education (KDU-CARE)</t>
-  </si>
-  <si>
     <t>Project 4/4-1.webp</t>
   </si>
   <si>
@@ -771,10 +759,6 @@
   </si>
   <si>
     <t>HYDRATech: Local Nanocoating Production</t>
-  </si>
-  <si>
-    <t>1,300+ Applicants at Entry to Semi-Finalists:
-IEEE Innovation Nation Sri Lanka (2021)</t>
   </si>
   <si>
     <t>Entrepreneurship</t>
@@ -1346,7 +1330,26 @@
     <t>Project 8/8-1.webp|Project 8/8-2.webp|Project 8/8-3.webp|Project 8/8-4.webp</t>
   </si>
   <si>
-    <t>Coming soon…</t>
+    <t>To build hyper-precise navigation systems without relying on GPS, we need sensors that measure microscopic forces. On Earth, gravity creates a wall: laser-trapped particles sag and drop out in less than a millisecond. So how do we break this limit without losing our payload every time? Team Aerolite set its scope to directly tackle this bottleneck with Project HALO. By pairing an electrical safety net with a precision laser trap under autonomous FPGA control, we've conceptualized a novel hybrid architecture that extends measurement windows $10^6\times$ for satellite navigation and Earth observation (TRL 2–3).</t>
+  </si>
+  <si>
+    <t>Semi-Finalists | 1,300+ Applicants at Entry:
+IEEE Innovation Nation Sri Lanka (2021)</t>
+  </si>
+  <si>
+    <t>Qualified to Next Round | Ongoing... | Results Announced Late 2026</t>
+  </si>
+  <si>
+    <t>Winner: EIIS x Airbus Annual Space Entrepreneurship Challenge | Space Debris Mitigation</t>
+  </si>
+  <si>
+    <t>Numeric Approach (CFD) | Best Poster Presentation | International Research Conference (2023)</t>
+  </si>
+  <si>
+    <t>Numeric Approach (CFD) | Best Research Project (2024), Department of Aeronautical Engineering</t>
+  </si>
+  <si>
+    <t>Experimental Approach (Lab) | Grant of LKR 1Mn Approved | Combinatorial Advanced Research &amp; Education (KDU-CARE)</t>
   </si>
 </sst>
 </file>
@@ -3192,22 +3195,25 @@
         <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>418</v>
+        <v>413</v>
       </c>
       <c r="C2" t="s">
-        <v>428</v>
+        <v>425</v>
+      </c>
+      <c r="D2" t="s">
+        <v>423</v>
       </c>
       <c r="E2" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="F2" t="s">
-        <v>426</v>
+        <v>421</v>
       </c>
       <c r="G2" t="s">
-        <v>427</v>
+        <v>422</v>
       </c>
       <c r="H2" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
@@ -3218,22 +3224,22 @@
         <v>219</v>
       </c>
       <c r="C3" t="s">
+        <v>426</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>416</v>
+      </c>
+      <c r="E3" t="s">
         <v>220</v>
       </c>
-      <c r="D3" s="1" t="s">
-        <v>421</v>
-      </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>221</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>222</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>223</v>
-      </c>
-      <c r="H3" t="s">
-        <v>224</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
@@ -3241,25 +3247,25 @@
         <v>6</v>
       </c>
       <c r="B4" t="s">
+        <v>224</v>
+      </c>
+      <c r="C4" t="s">
+        <v>427</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>417</v>
+      </c>
+      <c r="E4" t="s">
+        <v>220</v>
+      </c>
+      <c r="F4" t="s">
         <v>225</v>
       </c>
-      <c r="C4" t="s">
+      <c r="G4" t="s">
         <v>226</v>
       </c>
-      <c r="D4" s="1" t="s">
-        <v>422</v>
-      </c>
-      <c r="E4" t="s">
-        <v>221</v>
-      </c>
-      <c r="F4" t="s">
+      <c r="H4" t="s">
         <v>227</v>
-      </c>
-      <c r="G4" t="s">
-        <v>228</v>
-      </c>
-      <c r="H4" t="s">
-        <v>229</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.35">
@@ -3267,25 +3273,25 @@
         <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>419</v>
+        <v>414</v>
       </c>
       <c r="C5" t="s">
-        <v>230</v>
+        <v>428</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>423</v>
+        <v>418</v>
       </c>
       <c r="E5" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="F5" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="G5" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="H5" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
@@ -3293,25 +3299,25 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>420</v>
+        <v>415</v>
       </c>
       <c r="C6" t="s">
-        <v>233</v>
+        <v>429</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>424</v>
+        <v>419</v>
       </c>
       <c r="E6" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="F6" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="G6" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="H6" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.35">
@@ -3319,22 +3325,22 @@
         <v>3</v>
       </c>
       <c r="B7" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="C7" t="s">
-        <v>236</v>
+        <v>232</v>
       </c>
       <c r="E7" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="F7" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="G7" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="H7" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.35">
@@ -3342,22 +3348,22 @@
         <v>2</v>
       </c>
       <c r="B8" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="C8" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
       <c r="E8" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="F8" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="G8" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="H8" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.35">
@@ -3365,25 +3371,25 @@
         <v>1</v>
       </c>
       <c r="B9" t="s">
-        <v>242</v>
-      </c>
-      <c r="C9" t="s">
-        <v>243</v>
+        <v>238</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>424</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>425</v>
+        <v>420</v>
       </c>
       <c r="E9" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="F9" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="G9" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="H9" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
     </row>
   </sheetData>
@@ -3414,22 +3420,22 @@
         <v>194</v>
       </c>
       <c r="C1" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="D1" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
       <c r="E1" t="s">
         <v>217</v>
       </c>
       <c r="F1" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="G1" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="H1" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="I1" t="s">
         <v>22</v>
@@ -3440,10 +3446,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>252</v>
+        <v>247</v>
       </c>
       <c r="C2" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="E2" t="str">
         <f t="shared" ref="E2:E33" si="0">"thumbs/" &amp; B2 &amp; ".webp"</f>
@@ -3454,13 +3460,13 @@
         <v>pdfs/Master of Arts - Space Entrepreneurship.pdf</v>
       </c>
       <c r="G2" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="H2" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="I2" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.35">
@@ -3468,10 +3474,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="C3" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="E3" t="str">
         <f t="shared" si="0"/>
@@ -3482,10 +3488,10 @@
         <v>pdfs/Acceptance Letter - EIIS.pdf</v>
       </c>
       <c r="G3" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="H3" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.35">
@@ -3493,13 +3499,13 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="C4" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="D4" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
       <c r="E4" t="str">
         <f t="shared" si="0"/>
@@ -3510,13 +3516,13 @@
         <v>pdfs/Digitalisation in Aeronautics.pdf</v>
       </c>
       <c r="G4" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="H4" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="I4" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.35">
@@ -3524,13 +3530,13 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>261</v>
+        <v>256</v>
       </c>
       <c r="C5" t="s">
+        <v>252</v>
+      </c>
+      <c r="D5" t="s">
         <v>257</v>
-      </c>
-      <c r="D5" t="s">
-        <v>262</v>
       </c>
       <c r="E5" t="str">
         <f t="shared" si="0"/>
@@ -3541,13 +3547,13 @@
         <v>pdfs/Digitalisation in Space Research.pdf</v>
       </c>
       <c r="G5" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="H5" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="I5" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.35">
@@ -3555,13 +3561,13 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="C6" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="D6" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="E6" t="str">
         <f t="shared" si="0"/>
@@ -3572,13 +3578,13 @@
         <v>pdfs/Digitalisation in the Aerospace Industry.pdf</v>
       </c>
       <c r="G6" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="H6" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="I6" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.35">
@@ -3586,13 +3592,13 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="C7" t="s">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="D7" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="E7" t="str">
         <f t="shared" si="0"/>
@@ -3603,10 +3609,10 @@
         <v>pdfs/Aerospace Materials.pdf</v>
       </c>
       <c r="G7" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="I7" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.35">
@@ -3614,13 +3620,13 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="C8" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="D8" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="E8" t="str">
         <f t="shared" si="0"/>
@@ -3631,10 +3637,10 @@
         <v>pdfs/Robotics - Aerial Robotics.pdf</v>
       </c>
       <c r="G8" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="I8" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.35">
@@ -3642,10 +3648,10 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>271</v>
+        <v>266</v>
       </c>
       <c r="C9" t="s">
-        <v>272</v>
+        <v>267</v>
       </c>
       <c r="E9" t="str">
         <f t="shared" si="0"/>
@@ -3656,7 +3662,7 @@
         <v>pdfs/Best Research Project.pdf</v>
       </c>
       <c r="I9" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.35">
@@ -3664,10 +3670,10 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="C10" t="s">
-        <v>274</v>
+        <v>269</v>
       </c>
       <c r="E10" t="str">
         <f t="shared" si="0"/>
@@ -3678,10 +3684,10 @@
         <v>pdfs/Best Poster Presentation.pdf</v>
       </c>
       <c r="G10" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="I10" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.35">
@@ -3689,10 +3695,10 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="C11" t="s">
-        <v>274</v>
+        <v>269</v>
       </c>
       <c r="E11" t="str">
         <f t="shared" si="0"/>
@@ -3703,10 +3709,10 @@
         <v>pdfs/Paper Presentation at IRC.pdf</v>
       </c>
       <c r="G11" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="I11" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.35">
@@ -3714,10 +3720,10 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>276</v>
+        <v>271</v>
       </c>
       <c r="C12" t="s">
-        <v>272</v>
+        <v>267</v>
       </c>
       <c r="E12" t="str">
         <f t="shared" si="0"/>
@@ -3728,13 +3734,13 @@
         <v>pdfs/BSc. (Hons) Aeronautical Engineering.pdf</v>
       </c>
       <c r="G12" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="H12" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
       <c r="I12" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.35">
@@ -3742,7 +3748,7 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>278</v>
+        <v>273</v>
       </c>
       <c r="C13" t="s">
         <v>161</v>
@@ -3756,13 +3762,13 @@
         <v>pdfs/Chairperson - SEDS SL.pdf</v>
       </c>
       <c r="G13" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="H13" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
       <c r="I13" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.35">
@@ -3770,10 +3776,10 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>279</v>
+        <v>274</v>
       </c>
       <c r="C14" t="s">
-        <v>272</v>
+        <v>267</v>
       </c>
       <c r="E14" t="str">
         <f t="shared" si="0"/>
@@ -3784,10 +3790,10 @@
         <v>pdfs/President - SEDS KDU.pdf</v>
       </c>
       <c r="G14" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="I14" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.35">
@@ -3795,7 +3801,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="C15" t="s">
         <v>166</v>
@@ -3809,10 +3815,10 @@
         <v>pdfs/Service Letter.pdf</v>
       </c>
       <c r="G15" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="I15" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.35">
@@ -3820,13 +3826,13 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>281</v>
+        <v>276</v>
       </c>
       <c r="C16" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
       <c r="D16" t="s">
-        <v>283</v>
+        <v>278</v>
       </c>
       <c r="E16" t="str">
         <f t="shared" si="0"/>
@@ -3837,10 +3843,10 @@
         <v>pdfs/Semi-Finalists - IEEE INSL 2021.pdf</v>
       </c>
       <c r="G16" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
       <c r="I16" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.35">
@@ -3848,10 +3854,10 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
       <c r="C17" t="s">
-        <v>272</v>
+        <v>267</v>
       </c>
       <c r="E17" t="str">
         <f t="shared" si="0"/>
@@ -3862,10 +3868,10 @@
         <v>pdfs/Inter-Faculty Cricket (2022).pdf</v>
       </c>
       <c r="G17" t="s">
-        <v>286</v>
+        <v>281</v>
       </c>
       <c r="I17" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.35">
@@ -3873,10 +3879,10 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
       <c r="C18" t="s">
-        <v>272</v>
+        <v>267</v>
       </c>
       <c r="E18" t="str">
         <f t="shared" si="0"/>
@@ -3887,10 +3893,10 @@
         <v>pdfs/Inter-Faculty Cricket (2023).pdf</v>
       </c>
       <c r="G18" t="s">
-        <v>286</v>
+        <v>281</v>
       </c>
       <c r="I18" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.35">
@@ -3898,10 +3904,10 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>288</v>
+        <v>283</v>
       </c>
       <c r="C19" t="s">
-        <v>272</v>
+        <v>267</v>
       </c>
       <c r="E19" t="str">
         <f t="shared" si="0"/>
@@ -3912,10 +3918,10 @@
         <v>pdfs/Leadership Program (2020).pdf</v>
       </c>
       <c r="G19" t="s">
-        <v>289</v>
+        <v>284</v>
       </c>
       <c r="I19" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.35">
@@ -3923,10 +3929,10 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>290</v>
+        <v>285</v>
       </c>
       <c r="C20" t="s">
-        <v>272</v>
+        <v>267</v>
       </c>
       <c r="E20" t="str">
         <f t="shared" si="0"/>
@@ -3937,10 +3943,10 @@
         <v>pdfs/Leadership Program (2017).pdf</v>
       </c>
       <c r="G20" t="s">
-        <v>289</v>
+        <v>284</v>
       </c>
       <c r="I20" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.35">
@@ -3948,13 +3954,13 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>291</v>
+        <v>286</v>
       </c>
       <c r="C21" t="s">
-        <v>292</v>
+        <v>287</v>
       </c>
       <c r="D21" t="s">
-        <v>293</v>
+        <v>288</v>
       </c>
       <c r="E21" t="str">
         <f t="shared" si="0"/>
@@ -3965,13 +3971,13 @@
         <v>pdfs/Foundations of Project Management.pdf</v>
       </c>
       <c r="G21" t="s">
+        <v>284</v>
+      </c>
+      <c r="H21" t="s">
         <v>289</v>
       </c>
-      <c r="H21" t="s">
-        <v>294</v>
-      </c>
       <c r="I21" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.35">
@@ -3979,13 +3985,13 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>295</v>
+        <v>290</v>
       </c>
       <c r="C22" t="s">
-        <v>292</v>
+        <v>287</v>
       </c>
       <c r="D22" t="s">
-        <v>296</v>
+        <v>291</v>
       </c>
       <c r="E22" t="str">
         <f t="shared" si="0"/>
@@ -3996,13 +4002,13 @@
         <v>pdfs/Project Initiation - Starting a Successful Project.pdf</v>
       </c>
       <c r="G22" t="s">
+        <v>284</v>
+      </c>
+      <c r="H22" t="s">
         <v>289</v>
       </c>
-      <c r="H22" t="s">
-        <v>294</v>
-      </c>
       <c r="I22" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.35">
@@ -4010,13 +4016,13 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>297</v>
+        <v>292</v>
       </c>
       <c r="C23" t="s">
-        <v>292</v>
+        <v>287</v>
       </c>
       <c r="D23" t="s">
-        <v>298</v>
+        <v>293</v>
       </c>
       <c r="E23" t="str">
         <f t="shared" si="0"/>
@@ -4027,13 +4033,13 @@
         <v>pdfs/Project Planning - Putting It All Together.pdf</v>
       </c>
       <c r="G23" t="s">
+        <v>284</v>
+      </c>
+      <c r="H23" t="s">
         <v>289</v>
       </c>
-      <c r="H23" t="s">
-        <v>294</v>
-      </c>
       <c r="I23" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.35">
@@ -4041,13 +4047,13 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>299</v>
+        <v>294</v>
       </c>
       <c r="C24" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="D24" t="s">
-        <v>300</v>
+        <v>295</v>
       </c>
       <c r="E24" t="str">
         <f t="shared" si="0"/>
@@ -4058,10 +4064,10 @@
         <v>pdfs/Introduction to Marketing.pdf</v>
       </c>
       <c r="G24" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
       <c r="I24" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.35">
@@ -4069,10 +4075,10 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>301</v>
+        <v>296</v>
       </c>
       <c r="C25" t="s">
-        <v>292</v>
+        <v>287</v>
       </c>
       <c r="E25" t="str">
         <f t="shared" si="0"/>
@@ -4083,10 +4089,10 @@
         <v>pdfs/Fundamentals of Digital Marketing.pdf</v>
       </c>
       <c r="G25" t="s">
-        <v>302</v>
+        <v>297</v>
       </c>
       <c r="I25" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.35">
@@ -4094,13 +4100,13 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>303</v>
+        <v>298</v>
       </c>
       <c r="C26" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="D26" t="s">
-        <v>305</v>
+        <v>300</v>
       </c>
       <c r="E26" t="str">
         <f t="shared" si="0"/>
@@ -4111,13 +4117,13 @@
         <v>pdfs/Claude 101.pdf</v>
       </c>
       <c r="G26" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="H26" t="s">
-        <v>307</v>
+        <v>302</v>
       </c>
       <c r="I26" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.35">
@@ -4125,13 +4131,13 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>308</v>
+        <v>303</v>
       </c>
       <c r="C27" t="s">
+        <v>299</v>
+      </c>
+      <c r="D27" t="s">
         <v>304</v>
-      </c>
-      <c r="D27" t="s">
-        <v>309</v>
       </c>
       <c r="E27" t="str">
         <f t="shared" si="0"/>
@@ -4142,13 +4148,13 @@
         <v>pdfs/Claude Code 101.pdf</v>
       </c>
       <c r="G27" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="H27" t="s">
-        <v>307</v>
+        <v>302</v>
       </c>
       <c r="I27" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.35">
@@ -4156,13 +4162,13 @@
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>310</v>
+        <v>305</v>
       </c>
       <c r="C28" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="D28" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="E28" t="str">
         <f t="shared" si="0"/>
@@ -4173,13 +4179,13 @@
         <v>pdfs/Claude Platform 101.pdf</v>
       </c>
       <c r="G28" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="H28" t="s">
-        <v>307</v>
+        <v>302</v>
       </c>
       <c r="I28" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.35">
@@ -4187,13 +4193,13 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>312</v>
+        <v>307</v>
       </c>
       <c r="C29" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="D29" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
       <c r="E29" t="str">
         <f t="shared" si="0"/>
@@ -4204,13 +4210,13 @@
         <v>pdfs/Introduction to Claude Cowork.pdf</v>
       </c>
       <c r="G29" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="H29" t="s">
-        <v>307</v>
+        <v>302</v>
       </c>
       <c r="I29" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.35">
@@ -4218,13 +4224,13 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>314</v>
+        <v>309</v>
       </c>
       <c r="C30" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="D30" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="E30" t="str">
         <f t="shared" si="0"/>
@@ -4235,13 +4241,13 @@
         <v>pdfs/Claude Code in Action.pdf</v>
       </c>
       <c r="G30" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="H30" t="s">
-        <v>307</v>
+        <v>302</v>
       </c>
       <c r="I30" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.35">
@@ -4249,13 +4255,13 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>316</v>
+        <v>311</v>
       </c>
       <c r="C31" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="D31" t="s">
-        <v>317</v>
+        <v>312</v>
       </c>
       <c r="E31" t="str">
         <f t="shared" si="0"/>
@@ -4266,13 +4272,13 @@
         <v>pdfs/AI Fluency - Frameworks &amp; Foundations.pdf</v>
       </c>
       <c r="G31" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="H31" t="s">
-        <v>307</v>
+        <v>302</v>
       </c>
       <c r="I31" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.35">
@@ -4280,13 +4286,13 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>318</v>
+        <v>313</v>
       </c>
       <c r="C32" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="D32" t="s">
-        <v>319</v>
+        <v>314</v>
       </c>
       <c r="E32" t="str">
         <f t="shared" si="0"/>
@@ -4297,13 +4303,13 @@
         <v>pdfs/Introduction to Model Context Protocol.pdf</v>
       </c>
       <c r="G32" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="H32" t="s">
-        <v>307</v>
+        <v>302</v>
       </c>
       <c r="I32" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.35">
@@ -4311,13 +4317,13 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>320</v>
+        <v>315</v>
       </c>
       <c r="C33" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="D33" t="s">
-        <v>321</v>
+        <v>316</v>
       </c>
       <c r="E33" t="str">
         <f t="shared" si="0"/>
@@ -4328,13 +4334,13 @@
         <v>pdfs/Model Context Protocol - Advanced Topics.pdf</v>
       </c>
       <c r="G33" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="H33" t="s">
-        <v>307</v>
+        <v>302</v>
       </c>
       <c r="I33" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.35">
@@ -4342,13 +4348,13 @@
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>322</v>
+        <v>317</v>
       </c>
       <c r="C34" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="D34" t="s">
-        <v>323</v>
+        <v>318</v>
       </c>
       <c r="E34" t="str">
         <f t="shared" ref="E34:E52" si="2">"thumbs/" &amp; B34 &amp; ".webp"</f>
@@ -4359,13 +4365,13 @@
         <v>pdfs/AI Fluency for Educators.pdf</v>
       </c>
       <c r="G34" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="H34" t="s">
-        <v>307</v>
+        <v>302</v>
       </c>
       <c r="I34" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.35">
@@ -4373,13 +4379,13 @@
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
       <c r="C35" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="D35" t="s">
-        <v>325</v>
+        <v>320</v>
       </c>
       <c r="E35" t="str">
         <f t="shared" si="2"/>
@@ -4390,13 +4396,13 @@
         <v>pdfs/AI Fluency for Students.pdf</v>
       </c>
       <c r="G35" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="H35" t="s">
-        <v>307</v>
+        <v>302</v>
       </c>
       <c r="I35" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.35">
@@ -4404,13 +4410,13 @@
         <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>326</v>
+        <v>321</v>
       </c>
       <c r="C36" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="D36" t="s">
-        <v>327</v>
+        <v>322</v>
       </c>
       <c r="E36" t="str">
         <f t="shared" si="2"/>
@@ -4421,13 +4427,13 @@
         <v>pdfs/Teaching the AI Fluency Framework.pdf</v>
       </c>
       <c r="G36" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="H36" t="s">
-        <v>307</v>
+        <v>302</v>
       </c>
       <c r="I36" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.35">
@@ -4435,13 +4441,13 @@
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>328</v>
+        <v>323</v>
       </c>
       <c r="C37" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="D37" t="s">
-        <v>329</v>
+        <v>324</v>
       </c>
       <c r="E37" t="str">
         <f t="shared" si="2"/>
@@ -4452,13 +4458,13 @@
         <v>pdfs/AI Fluency for Non-Profits.pdf</v>
       </c>
       <c r="G37" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="H37" t="s">
-        <v>307</v>
+        <v>302</v>
       </c>
       <c r="I37" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.35">
@@ -4466,13 +4472,13 @@
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>330</v>
+        <v>325</v>
       </c>
       <c r="C38" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="D38" t="s">
-        <v>331</v>
+        <v>326</v>
       </c>
       <c r="E38" t="str">
         <f t="shared" si="2"/>
@@ -4483,13 +4489,13 @@
         <v>pdfs/AI Fluency for Small Businesses.pdf</v>
       </c>
       <c r="G38" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="H38" t="s">
-        <v>307</v>
+        <v>302</v>
       </c>
       <c r="I38" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.35">
@@ -4497,13 +4503,13 @@
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>332</v>
+        <v>327</v>
       </c>
       <c r="C39" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="D39" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="E39" t="str">
         <f t="shared" si="2"/>
@@ -4514,13 +4520,13 @@
         <v>pdfs/Introduction to Agent Skills.pdf</v>
       </c>
       <c r="G39" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="H39" t="s">
-        <v>307</v>
+        <v>302</v>
       </c>
       <c r="I39" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.35">
@@ -4528,13 +4534,13 @@
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>334</v>
+        <v>329</v>
       </c>
       <c r="C40" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="D40" t="s">
-        <v>335</v>
+        <v>330</v>
       </c>
       <c r="E40" t="str">
         <f t="shared" si="2"/>
@@ -4545,13 +4551,13 @@
         <v>pdfs/Introduction to Sub-Agents.pdf</v>
       </c>
       <c r="G40" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="H40" t="s">
-        <v>307</v>
+        <v>302</v>
       </c>
       <c r="I40" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.35">
@@ -4559,13 +4565,13 @@
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>336</v>
+        <v>331</v>
       </c>
       <c r="C41" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="D41" t="s">
-        <v>337</v>
+        <v>332</v>
       </c>
       <c r="E41" t="str">
         <f t="shared" si="2"/>
@@ -4576,13 +4582,13 @@
         <v>pdfs/AI Capabilities &amp; Limitations.pdf</v>
       </c>
       <c r="G41" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="H41" t="s">
-        <v>307</v>
+        <v>302</v>
       </c>
       <c r="I41" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.35">
@@ -4590,13 +4596,13 @@
         <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
       <c r="C42" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="D42" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
       <c r="E42" t="str">
         <f t="shared" si="2"/>
@@ -4607,13 +4613,13 @@
         <v>pdfs/Claude with Anthropic API.pdf</v>
       </c>
       <c r="G42" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="H42" t="s">
-        <v>307</v>
+        <v>302</v>
       </c>
       <c r="I42" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.35">
@@ -4621,13 +4627,13 @@
         <v>42</v>
       </c>
       <c r="B43" t="s">
-        <v>340</v>
+        <v>335</v>
       </c>
       <c r="C43" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="D43" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="E43" t="str">
         <f t="shared" si="2"/>
@@ -4638,13 +4644,13 @@
         <v>pdfs/Claude with Google Vertex AI.pdf</v>
       </c>
       <c r="G43" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="H43" t="s">
-        <v>307</v>
+        <v>302</v>
       </c>
       <c r="I43" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.35">
@@ -4652,13 +4658,13 @@
         <v>43</v>
       </c>
       <c r="B44" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="C44" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="D44" t="s">
-        <v>343</v>
+        <v>338</v>
       </c>
       <c r="E44" t="str">
         <f t="shared" si="2"/>
@@ -4669,13 +4675,13 @@
         <v>pdfs/Claude with Amazon Bedrock.pdf</v>
       </c>
       <c r="G44" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="H44" t="s">
-        <v>307</v>
+        <v>302</v>
       </c>
       <c r="I44" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.35">
@@ -4683,13 +4689,13 @@
         <v>44</v>
       </c>
       <c r="B45" t="s">
-        <v>344</v>
+        <v>339</v>
       </c>
       <c r="C45" t="s">
-        <v>345</v>
+        <v>340</v>
       </c>
       <c r="D45" t="s">
-        <v>346</v>
+        <v>341</v>
       </c>
       <c r="E45" t="str">
         <f t="shared" si="2"/>
@@ -4700,10 +4706,10 @@
         <v>pdfs/Getting Started with Python.pdf</v>
       </c>
       <c r="G45" t="s">
-        <v>347</v>
+        <v>342</v>
       </c>
       <c r="I45" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.35">
@@ -4711,10 +4717,10 @@
         <v>45</v>
       </c>
       <c r="B46" t="s">
-        <v>348</v>
+        <v>343</v>
       </c>
       <c r="C46" t="s">
-        <v>349</v>
+        <v>344</v>
       </c>
       <c r="E46" t="str">
         <f t="shared" si="2"/>
@@ -4725,10 +4731,10 @@
         <v>pdfs/Gampaha District Cricket Team.pdf</v>
       </c>
       <c r="G46" t="s">
-        <v>286</v>
+        <v>281</v>
       </c>
       <c r="I46" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.35">
@@ -4736,7 +4742,7 @@
         <v>46</v>
       </c>
       <c r="B47" t="s">
-        <v>350</v>
+        <v>345</v>
       </c>
       <c r="C47" t="s">
         <v>196</v>
@@ -4750,10 +4756,10 @@
         <v>pdfs/Sports Colors - Cricket.pdf</v>
       </c>
       <c r="G47" t="s">
-        <v>286</v>
+        <v>281</v>
       </c>
       <c r="I47" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.35">
@@ -4761,10 +4767,10 @@
         <v>47</v>
       </c>
       <c r="B48" t="s">
-        <v>351</v>
+        <v>346</v>
       </c>
       <c r="C48" t="s">
-        <v>352</v>
+        <v>347</v>
       </c>
       <c r="E48" t="str">
         <f t="shared" si="2"/>
@@ -4775,10 +4781,10 @@
         <v>pdfs/All-Island U19 DIII Semi-Finalists (2019).pdf</v>
       </c>
       <c r="G48" t="s">
-        <v>286</v>
+        <v>281</v>
       </c>
       <c r="I48" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.35">
@@ -4786,7 +4792,7 @@
         <v>48</v>
       </c>
       <c r="B49" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
       <c r="C49" t="s">
         <v>196</v>
@@ -4800,10 +4806,10 @@
         <v>pdfs/School Leaving Certificate.pdf</v>
       </c>
       <c r="G49" t="s">
-        <v>354</v>
+        <v>349</v>
       </c>
       <c r="I49" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.35">
@@ -4811,7 +4817,7 @@
         <v>49</v>
       </c>
       <c r="B50" t="s">
-        <v>355</v>
+        <v>350</v>
       </c>
       <c r="C50" t="s">
         <v>196</v>
@@ -4825,10 +4831,10 @@
         <v>pdfs/Character Certificate.pdf</v>
       </c>
       <c r="G50" t="s">
-        <v>354</v>
+        <v>349</v>
       </c>
       <c r="I50" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.35">
@@ -4836,10 +4842,10 @@
         <v>50</v>
       </c>
       <c r="B51" t="s">
-        <v>356</v>
+        <v>351</v>
       </c>
       <c r="C51" t="s">
-        <v>357</v>
+        <v>352</v>
       </c>
       <c r="E51" t="str">
         <f t="shared" si="2"/>
@@ -4850,10 +4856,10 @@
         <v>pdfs/Advanced Level Results.pdf</v>
       </c>
       <c r="G51" t="s">
-        <v>354</v>
+        <v>349</v>
       </c>
       <c r="I51" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.35">
@@ -4861,10 +4867,10 @@
         <v>51</v>
       </c>
       <c r="B52" t="s">
-        <v>358</v>
+        <v>353</v>
       </c>
       <c r="C52" t="s">
-        <v>359</v>
+        <v>354</v>
       </c>
       <c r="E52" t="str">
         <f t="shared" si="2"/>
@@ -4875,10 +4881,10 @@
         <v>pdfs/IGCSE OL Results.pdf</v>
       </c>
       <c r="G52" t="s">
-        <v>354</v>
+        <v>349</v>
       </c>
       <c r="I52" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
     </row>
   </sheetData>
@@ -4908,7 +4914,7 @@
         <v>217</v>
       </c>
       <c r="E1" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
       <c r="F1" t="s">
         <v>216</v>
@@ -4922,22 +4928,22 @@
         <v>14</v>
       </c>
       <c r="B2" t="s">
-        <v>415</v>
+        <v>410</v>
       </c>
       <c r="C2" t="s">
-        <v>414</v>
+        <v>409</v>
       </c>
       <c r="D2" t="s">
-        <v>361</v>
+        <v>356</v>
       </c>
       <c r="E2" t="s">
-        <v>362</v>
+        <v>357</v>
       </c>
       <c r="F2" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G2" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
@@ -4945,22 +4951,22 @@
         <v>13</v>
       </c>
       <c r="B3" t="s">
-        <v>363</v>
+        <v>358</v>
       </c>
       <c r="C3" t="s">
-        <v>364</v>
+        <v>359</v>
       </c>
       <c r="D3" t="s">
-        <v>365</v>
+        <v>360</v>
       </c>
       <c r="E3" t="s">
-        <v>366</v>
+        <v>361</v>
       </c>
       <c r="F3" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="G3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
@@ -4968,22 +4974,22 @@
         <v>12</v>
       </c>
       <c r="B4" t="s">
-        <v>416</v>
+        <v>411</v>
       </c>
       <c r="C4" t="s">
-        <v>368</v>
+        <v>363</v>
       </c>
       <c r="D4" t="s">
-        <v>369</v>
+        <v>364</v>
       </c>
       <c r="E4" t="s">
-        <v>370</v>
+        <v>365</v>
       </c>
       <c r="F4" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G4" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
@@ -4991,22 +4997,22 @@
         <v>11</v>
       </c>
       <c r="B5" t="s">
-        <v>371</v>
+        <v>366</v>
       </c>
       <c r="C5" t="s">
-        <v>372</v>
+        <v>367</v>
       </c>
       <c r="D5" t="s">
-        <v>373</v>
+        <v>368</v>
       </c>
       <c r="E5" t="s">
-        <v>374</v>
+        <v>369</v>
       </c>
       <c r="F5" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G5" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
@@ -5014,22 +5020,22 @@
         <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>417</v>
+        <v>412</v>
       </c>
       <c r="C6" t="s">
-        <v>375</v>
+        <v>370</v>
       </c>
       <c r="D6" t="s">
-        <v>376</v>
+        <v>371</v>
       </c>
       <c r="E6" t="s">
-        <v>377</v>
+        <v>372</v>
       </c>
       <c r="F6" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G6" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
@@ -5037,22 +5043,22 @@
         <v>9</v>
       </c>
       <c r="B7" t="s">
-        <v>378</v>
+        <v>373</v>
       </c>
       <c r="C7" t="s">
-        <v>379</v>
+        <v>374</v>
       </c>
       <c r="D7" t="s">
-        <v>380</v>
+        <v>375</v>
       </c>
       <c r="E7" t="s">
-        <v>381</v>
+        <v>376</v>
       </c>
       <c r="F7" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G7" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
@@ -5060,22 +5066,22 @@
         <v>8</v>
       </c>
       <c r="B8" t="s">
-        <v>382</v>
+        <v>377</v>
       </c>
       <c r="C8" t="s">
-        <v>383</v>
+        <v>378</v>
       </c>
       <c r="D8" t="s">
-        <v>384</v>
+        <v>379</v>
       </c>
       <c r="E8" t="s">
-        <v>385</v>
+        <v>380</v>
       </c>
       <c r="F8" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G8" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
@@ -5083,22 +5089,22 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="C9" t="s">
-        <v>387</v>
+        <v>382</v>
       </c>
       <c r="D9" t="s">
-        <v>388</v>
+        <v>383</v>
       </c>
       <c r="E9" t="s">
-        <v>389</v>
+        <v>384</v>
       </c>
       <c r="F9" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G9" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.35">
@@ -5106,22 +5112,22 @@
         <v>6</v>
       </c>
       <c r="B10" t="s">
-        <v>390</v>
+        <v>385</v>
       </c>
       <c r="C10" t="s">
-        <v>391</v>
+        <v>386</v>
       </c>
       <c r="D10" t="s">
-        <v>392</v>
+        <v>387</v>
       </c>
       <c r="E10" t="s">
-        <v>393</v>
+        <v>388</v>
       </c>
       <c r="F10" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="G10" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
@@ -5129,22 +5135,22 @@
         <v>5</v>
       </c>
       <c r="B11" t="s">
-        <v>394</v>
+        <v>389</v>
       </c>
       <c r="C11" t="s">
-        <v>395</v>
+        <v>390</v>
       </c>
       <c r="D11" t="s">
-        <v>396</v>
+        <v>391</v>
       </c>
       <c r="E11" t="s">
-        <v>397</v>
+        <v>392</v>
       </c>
       <c r="F11" t="s">
-        <v>286</v>
+        <v>281</v>
       </c>
       <c r="G11" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.35">
@@ -5152,22 +5158,22 @@
         <v>4</v>
       </c>
       <c r="B12" t="s">
-        <v>398</v>
+        <v>393</v>
       </c>
       <c r="C12" t="s">
-        <v>399</v>
+        <v>394</v>
       </c>
       <c r="D12" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
       <c r="E12" t="s">
-        <v>401</v>
+        <v>396</v>
       </c>
       <c r="F12" t="s">
-        <v>402</v>
+        <v>397</v>
       </c>
       <c r="G12" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.35">
@@ -5175,22 +5181,22 @@
         <v>3</v>
       </c>
       <c r="B13" t="s">
-        <v>403</v>
+        <v>398</v>
       </c>
       <c r="C13" t="s">
-        <v>404</v>
+        <v>399</v>
       </c>
       <c r="D13" t="s">
-        <v>405</v>
+        <v>400</v>
       </c>
       <c r="E13" t="s">
-        <v>406</v>
+        <v>401</v>
       </c>
       <c r="F13" t="s">
-        <v>286</v>
+        <v>281</v>
       </c>
       <c r="G13" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.35">
@@ -5198,22 +5204,22 @@
         <v>2</v>
       </c>
       <c r="B14" t="s">
-        <v>407</v>
+        <v>402</v>
       </c>
       <c r="C14" t="s">
-        <v>408</v>
+        <v>403</v>
       </c>
       <c r="D14" t="s">
-        <v>409</v>
+        <v>404</v>
       </c>
       <c r="E14" t="s">
-        <v>410</v>
+        <v>405</v>
       </c>
       <c r="F14" t="s">
-        <v>286</v>
+        <v>281</v>
       </c>
       <c r="G14" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.35">
@@ -5221,22 +5227,22 @@
         <v>1</v>
       </c>
       <c r="B15" t="s">
-        <v>411</v>
+        <v>406</v>
       </c>
       <c r="C15" t="s">
-        <v>412</v>
+        <v>407</v>
       </c>
       <c r="D15" t="s">
-        <v>413</v>
+        <v>408</v>
       </c>
       <c r="E15" t="s">
-        <v>362</v>
+        <v>357</v>
       </c>
       <c r="F15" t="s">
-        <v>286</v>
+        <v>281</v>
       </c>
       <c r="G15" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
   </sheetData>

</xml_diff>